<commit_message>
Fix Vnstock CLI runtime dependencies
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5a4ffa9fae1048b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONNECTION_FLOW" sheetId="2" r:id="R6064429075984615"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUBLIC_MACRO" sheetId="3" r:id="R056c2111153d4555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_FALLBACK" sheetId="4" r:id="Ra8b0470d9943462b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="5" r:id="R11f1b4c162fc453c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rff396763d3e4491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONNECTION_FLOW" sheetId="2" r:id="R3358adb0dcd4442f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUBLIC_MACRO" sheetId="3" r:id="R930b531e9b314c0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_FALLBACK" sheetId="4" r:id="Ra6292ac162a4498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="5" r:id="R8cd0d9e6a9754e6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +43,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -65,6 +65,11 @@
         <x:fgColor rgb="FFFFFF00"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -73,7 +78,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -110,6 +115,15 @@
     <x:xf numFmtId="200" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -312,7 +326,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="94" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -398,6 +412,46 @@
       </x:c>
       <x:c r="B11" t="str">
         <x:v>Không hiển thị số phiên bản trên tiêu đề app.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="27" t="str">
+        <x:v>Hotfix</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>V6.6.1 Runtime Dependency Preflight</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="28" t="str">
+        <x:v>CLI dependency</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="str">
+        <x:v>requests&gt;=2.31,&lt;3 được khai báo trong requirements.txt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="28" t="str">
+        <x:v>CLI dependency</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="str">
+        <x:v>packaging&gt;=23,&lt;27 được khai báo trong requirements.txt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="28" t="str">
+        <x:v>Runtime guard</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="str">
+        <x:v>app.py tự kiểm tra và cài dependency bằng sys.executable -m pip nếu Cloud thiếu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="28" t="str">
+        <x:v>Mục tiêu</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="str">
+        <x:v>Ngăn lỗi ModuleNotFoundError: No module named 'requests' trước khi Vnstock CLI chạy.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Move Vnstock Bronze to production data pipeline
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,11 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rff396763d3e4491c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONNECTION_FLOW" sheetId="2" r:id="R3358adb0dcd4442f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUBLIC_MACRO" sheetId="3" r:id="R930b531e9b314c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_FALLBACK" sheetId="4" r:id="Ra6292ac162a4498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="5" r:id="R8cd0d9e6a9754e6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1d68d4850c344083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARCHITECTURE" sheetId="2" r:id="R9b409e88a5b049cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA_LINEAGE" sheetId="3" r:id="R087033fd8bcb4014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUBLIC_MACRO" sheetId="4" r:id="R2f2688c9726a4545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ACTUALS_BRONZE" sheetId="5" r:id="R953fb4ec5fb54a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_FALLBACK" sheetId="6" r:id="R7c86f5e79f5b45d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="7" r:id="R88b7bb628a014da5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="0.00%"/>
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="#,##0.00;[Red](#,##0.00);-"/>
+    <x:numFmt numFmtId="201" formatCode="0.00%;[Red](0.00%);-"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -42,8 +45,13 @@
       <x:color rgb="FF0000FF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -65,11 +73,6 @@
         <x:fgColor rgb="FFFFFF00"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF0B6E69"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -78,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -111,19 +114,16 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -327,7 +327,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="94" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="96" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -352,106 +352,82 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>API Key</x:v>
+        <x:v>Kiến trúc</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>VNSTOCK_API_KEY từ Streamlit Secrets.</x:v>
+        <x:v>Bronze acquisition tách khỏi Streamlit runtime.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Connect button</x:v>
+        <x:v>Bronze source</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Luôn hiện khi có API Key nhưng vnstock_data chưa sẵn sàng.</x:v>
+        <x:v>vnstock_data chạy trên máy/self-hosted runner ổn định.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Installer trigger</x:v>
+        <x:v>Streamlit</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Chỉ chạy sau thao tác người dùng.</x:v>
+        <x:v>Chỉ đọc CSV ACTUAL từ GitHub, không import vnstock_data.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Progress</x:v>
+        <x:v>Lợi ích</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>3 bước: kiểm key → installer → kiểm vnstock_data.</x:v>
+        <x:v>Không còn installer crash/rate-limit trong Streamlit.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Bronze guardrail</x:v>
+        <x:v>Tự động hóa</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Probe 3 mã/12s trước full-load.</x:v>
+        <x:v>REFRESH_BRONZE_AND_PUSH.bat hoặc GitHub self-hosted runner.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Free guardrail</x:v>
+        <x:v>Device policy</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Chỉ probe 3 mã; không full-load Guest.</x:v>
+        <x:v>Ưu tiên máy persistent để tránh tạo thiết bị mới ngoài ý muốn.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Circuit breaker</x:v>
+        <x:v>Actual bank file</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>Ngăn gọi API lặp lại trên rerun.</x:v>
+        <x:v>data/bank_actuals_bronze.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>UI branding</x:v>
+        <x:v>Actual macro files</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Không hiển thị số phiên bản trên tiêu đề app.</x:v>
+        <x:v>data/*_bronze.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Fallback</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>ASSUMPTION chỉ dùng khi ACTUAL thiếu.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="27" t="str">
-        <x:v>Hotfix</x:v>
-      </x:c>
-      <x:c r="B13" s="27" t="str">
-        <x:v>V6.6.1 Runtime Dependency Preflight</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="28" t="str">
-        <x:v>CLI dependency</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="str">
-        <x:v>requests&gt;=2.31,&lt;3 được khai báo trong requirements.txt.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="28" t="str">
-        <x:v>CLI dependency</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="str">
-        <x:v>packaging&gt;=23,&lt;27 được khai báo trong requirements.txt.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="28" t="str">
-        <x:v>Runtime guard</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="str">
-        <x:v>app.py tự kiểm tra và cài dependency bằng sys.executable -m pip nếu Cloud thiếu.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="28" t="str">
-        <x:v>Mục tiêu</x:v>
-      </x:c>
-      <x:c r="B17" s="28" t="str">
-        <x:v>Ngăn lỗi ModuleNotFoundError: No module named 'requests' trước khi Vnstock CLI chạy.</x:v>
+      <x:c r="A13" t="str">
+        <x:v>Production rule</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>ACTUAL luôn ghi đè ASSUMPTION theo ticker.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -467,17 +443,17 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>VNSTOCK BRONZE CONNECTION FLOW</x:v>
+        <x:v>PRODUCTION BRONZE DATA ARCHITECTURE</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -491,22 +467,22 @@
         <x:v>Step</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
-        <x:v>Condition</x:v>
+        <x:v>Environment</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
-        <x:v>User action</x:v>
+        <x:v>Component</x:v>
       </x:c>
       <x:c r="D3" s="10" t="str">
-        <x:v>Max time</x:v>
+        <x:v>Input</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
-        <x:v>Success</x:v>
+        <x:v>Output</x:v>
       </x:c>
       <x:c r="F3" s="10" t="str">
-        <x:v>Failure</x:v>
+        <x:v>Runs when</x:v>
       </x:c>
       <x:c r="G3" s="10" t="str">
-        <x:v>Fallback</x:v>
+        <x:v>Risk control</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -514,22 +490,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>API Key missing</x:v>
+        <x:v>Stable PC/server</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Enter API Key / add Secret</x:v>
+        <x:v>Vnstock Sponsor</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>N/A</x:v>
+        <x:v>API key/device activation</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>Key configured</x:v>
+        <x:v>vnstock_data ready</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>Stay Free</x:v>
+        <x:v>One-time</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>Free/Public</x:v>
+        <x:v>Persistent device</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -537,22 +513,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Key exists + Sponsor missing</x:v>
+        <x:v>Stable PC/server</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Click Kết nối Bronze</x:v>
+        <x:v>refresh_bronze.py</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>90 sec</x:v>
+        <x:v>vnstock_data</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>vnstock_data available</x:v>
+        <x:v>data/*.csv ACTUAL</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>Show detailed log</x:v>
+        <x:v>Manual/scheduled</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>Free/Public</x:v>
+        <x:v>0.25s pacing</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -560,22 +536,22 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Sponsor available</x:v>
+        <x:v>Git</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Probe 3 banks</x:v>
+        <x:v>Commit/push</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>12 sec</x:v>
+        <x:v>data/*.csv</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>&gt;=2 useful</x:v>
+        <x:v>Repository updated</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Open Bronze circuit</x:v>
+        <x:v>After refresh</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>Free</x:v>
+        <x:v>Only data tracked</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -583,22 +559,22 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Bronze probe passes</x:v>
+        <x:v>Streamlit Cloud</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Load remaining 17</x:v>
+        <x:v>app.py</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>20 sec</x:v>
+        <x:v>Repository CSV</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Use Bronze ACTUAL</x:v>
+        <x:v>Dashboard/model</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Use returned rows</x:v>
+        <x:v>On deploy/rerun</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>Fallback missing banks</x:v>
+        <x:v>No Vnstock API call</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -606,22 +582,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Free mode</x:v>
+        <x:v>Fallback</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Probe 3 banks only</x:v>
+        <x:v>bank assumptions</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>12 sec</x:v>
+        <x:v>Missing actual ticker</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Use Free probe</x:v>
+        <x:v>Complete model universe</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>Open Free circuit</x:v>
+        <x:v>Only if missing</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Explicit ASSUMPTION</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -629,22 +605,22 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Both unavailable</x:v>
+        <x:v>Automation</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>No user action</x:v>
+        <x:v>Self-hosted runner</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>0 sec</x:v>
+        <x:v>Stable PC/server</x:v>
       </x:c>
       <x:c r="E9" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Scheduled refresh</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>Use fallback</x:v>
+        <x:v>Weekdays</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>Public + Assumption</x:v>
+        <x:v>No ephemeral runner</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -656,6 +632,170 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>DATA LINEAGE</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="10" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>Source Mode</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>Data Type</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>File</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>Universe</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>Refresh</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>Used by</x:v>
+      </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>BRONZE</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>bank_actuals_bronze.csv</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>20 banks</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Local/self-hosted</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Bank stress</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Overrides fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>BRONZE</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>*_bronze.csv</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Macro</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Local/self-hosted</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>System liquidity</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Primary actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>PUBLIC</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>macro_public_snapshot.csv</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Macro snapshot</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Bundled</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>System dashboard</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Fallback macro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>bank_fallback_assumptions.csv</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>20 banks</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Bundled</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Missing tickers</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Never relabel as actual</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -704,7 +844,7 @@
       <x:c r="B4" t="str">
         <x:v>Tăng trưởng tín dụng YTD</x:v>
       </x:c>
-      <x:c r="C4" t="n">
+      <x:c r="C4" s="18" t="n">
         <x:v>7.41</x:v>
       </x:c>
       <x:c r="D4" t="str">
@@ -724,7 +864,7 @@
       <x:c r="B5" t="str">
         <x:v>Tăng trưởng huy động YTD</x:v>
       </x:c>
-      <x:c r="C5" t="n">
+      <x:c r="C5" s="18" t="n">
         <x:v>5.02</x:v>
       </x:c>
       <x:c r="D5" t="str">
@@ -744,7 +884,7 @@
       <x:c r="B6" t="str">
         <x:v>CPI YoY</x:v>
       </x:c>
-      <x:c r="C6" t="n">
+      <x:c r="C6" s="18" t="n">
         <x:v>4.69</x:v>
       </x:c>
       <x:c r="D6" t="str">
@@ -764,7 +904,7 @@
       <x:c r="B7" t="str">
         <x:v>Lạm phát cơ bản</x:v>
       </x:c>
-      <x:c r="C7" t="n">
+      <x:c r="C7" s="18" t="n">
         <x:v>4.12</x:v>
       </x:c>
       <x:c r="D7" t="str">
@@ -784,7 +924,7 @@
       <x:c r="B8" t="str">
         <x:v>GDP YoY</x:v>
       </x:c>
-      <x:c r="C8" t="n">
+      <x:c r="C8" s="18" t="n">
         <x:v>8.39</x:v>
       </x:c>
       <x:c r="D8" t="str">
@@ -804,7 +944,7 @@
       <x:c r="B9" t="str">
         <x:v>Cán cân thương mại</x:v>
       </x:c>
-      <x:c r="C9" t="n">
+      <x:c r="C9" s="18" t="n">
         <x:v>-16.65</x:v>
       </x:c>
       <x:c r="D9" t="str">
@@ -825,7 +965,756 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>BANK ACTUALS — BRONZE PIPELINE</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+      <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="10" t="str">
+        <x:v>Ticker</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>Period</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>LDR</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>CASA</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>InterbankDep</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>CreditDepositGap</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>NIM</x:v>
+      </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>Data Type</x:v>
+      </x:c>
+      <x:c r="I3" s="10" t="str">
+        <x:v>Source Mode</x:v>
+      </x:c>
+      <x:c r="J3" s="10" t="str">
+        <x:v>Retrieved At</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="C4" s="22"/>
+      <x:c r="D4" s="22"/>
+      <x:c r="E4" s="22"/>
+      <x:c r="F4" s="22"/>
+      <x:c r="G4" s="22"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="C5" s="22"/>
+      <x:c r="D5" s="22"/>
+      <x:c r="E5" s="22"/>
+      <x:c r="F5" s="22"/>
+      <x:c r="G5" s="22"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="C6" s="22"/>
+      <x:c r="D6" s="22"/>
+      <x:c r="E6" s="22"/>
+      <x:c r="F6" s="22"/>
+      <x:c r="G6" s="22"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="C7" s="22"/>
+      <x:c r="D7" s="22"/>
+      <x:c r="E7" s="22"/>
+      <x:c r="F7" s="22"/>
+      <x:c r="G7" s="22"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="C8" s="22"/>
+      <x:c r="D8" s="22"/>
+      <x:c r="E8" s="22"/>
+      <x:c r="F8" s="22"/>
+      <x:c r="G8" s="22"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="C9" s="22"/>
+      <x:c r="D9" s="22"/>
+      <x:c r="E9" s="22"/>
+      <x:c r="F9" s="22"/>
+      <x:c r="G9" s="22"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="C10" s="22"/>
+      <x:c r="D10" s="22"/>
+      <x:c r="E10" s="22"/>
+      <x:c r="F10" s="22"/>
+      <x:c r="G10" s="22"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="C11" s="22"/>
+      <x:c r="D11" s="22"/>
+      <x:c r="E11" s="22"/>
+      <x:c r="F11" s="22"/>
+      <x:c r="G11" s="22"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="C12" s="22"/>
+      <x:c r="D12" s="22"/>
+      <x:c r="E12" s="22"/>
+      <x:c r="F12" s="22"/>
+      <x:c r="G12" s="22"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="C13" s="22"/>
+      <x:c r="D13" s="22"/>
+      <x:c r="E13" s="22"/>
+      <x:c r="F13" s="22"/>
+      <x:c r="G13" s="22"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="C14" s="22"/>
+      <x:c r="D14" s="22"/>
+      <x:c r="E14" s="22"/>
+      <x:c r="F14" s="22"/>
+      <x:c r="G14" s="22"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="C15" s="22"/>
+      <x:c r="D15" s="22"/>
+      <x:c r="E15" s="22"/>
+      <x:c r="F15" s="22"/>
+      <x:c r="G15" s="22"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="C16" s="22"/>
+      <x:c r="D16" s="22"/>
+      <x:c r="E16" s="22"/>
+      <x:c r="F16" s="22"/>
+      <x:c r="G16" s="22"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="C17" s="22"/>
+      <x:c r="D17" s="22"/>
+      <x:c r="E17" s="22"/>
+      <x:c r="F17" s="22"/>
+      <x:c r="G17" s="22"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="C18" s="22"/>
+      <x:c r="D18" s="22"/>
+      <x:c r="E18" s="22"/>
+      <x:c r="F18" s="22"/>
+      <x:c r="G18" s="22"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="C19" s="22"/>
+      <x:c r="D19" s="22"/>
+      <x:c r="E19" s="22"/>
+      <x:c r="F19" s="22"/>
+      <x:c r="G19" s="22"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="C20" s="22"/>
+      <x:c r="D20" s="22"/>
+      <x:c r="E20" s="22"/>
+      <x:c r="F20" s="22"/>
+      <x:c r="G20" s="22"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="C21" s="22"/>
+      <x:c r="D21" s="22"/>
+      <x:c r="E21" s="22"/>
+      <x:c r="F21" s="22"/>
+      <x:c r="G21" s="22"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="C22" s="22"/>
+      <x:c r="D22" s="22"/>
+      <x:c r="E22" s="22"/>
+      <x:c r="F22" s="22"/>
+      <x:c r="G22" s="22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="C23" s="22"/>
+      <x:c r="D23" s="22"/>
+      <x:c r="E23" s="22"/>
+      <x:c r="F23" s="22"/>
+      <x:c r="G23" s="22"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="C24" s="22"/>
+      <x:c r="D24" s="22"/>
+      <x:c r="E24" s="22"/>
+      <x:c r="F24" s="22"/>
+      <x:c r="G24" s="22"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="C25" s="22"/>
+      <x:c r="D25" s="22"/>
+      <x:c r="E25" s="22"/>
+      <x:c r="F25" s="22"/>
+      <x:c r="G25" s="22"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="C26" s="22"/>
+      <x:c r="D26" s="22"/>
+      <x:c r="E26" s="22"/>
+      <x:c r="F26" s="22"/>
+      <x:c r="G26" s="22"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="C27" s="22"/>
+      <x:c r="D27" s="22"/>
+      <x:c r="E27" s="22"/>
+      <x:c r="F27" s="22"/>
+      <x:c r="G27" s="22"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="C28" s="22"/>
+      <x:c r="D28" s="22"/>
+      <x:c r="E28" s="22"/>
+      <x:c r="F28" s="22"/>
+      <x:c r="G28" s="22"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="C29" s="22"/>
+      <x:c r="D29" s="22"/>
+      <x:c r="E29" s="22"/>
+      <x:c r="F29" s="22"/>
+      <x:c r="G29" s="22"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="C30" s="22"/>
+      <x:c r="D30" s="22"/>
+      <x:c r="E30" s="22"/>
+      <x:c r="F30" s="22"/>
+      <x:c r="G30" s="22"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="C31" s="22"/>
+      <x:c r="D31" s="22"/>
+      <x:c r="E31" s="22"/>
+      <x:c r="F31" s="22"/>
+      <x:c r="G31" s="22"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="C32" s="22"/>
+      <x:c r="D32" s="22"/>
+      <x:c r="E32" s="22"/>
+      <x:c r="F32" s="22"/>
+      <x:c r="G32" s="22"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="C33" s="22"/>
+      <x:c r="D33" s="22"/>
+      <x:c r="E33" s="22"/>
+      <x:c r="F33" s="22"/>
+      <x:c r="G33" s="22"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="C34" s="22"/>
+      <x:c r="D34" s="22"/>
+      <x:c r="E34" s="22"/>
+      <x:c r="F34" s="22"/>
+      <x:c r="G34" s="22"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="C35" s="22"/>
+      <x:c r="D35" s="22"/>
+      <x:c r="E35" s="22"/>
+      <x:c r="F35" s="22"/>
+      <x:c r="G35" s="22"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="C36" s="22"/>
+      <x:c r="D36" s="22"/>
+      <x:c r="E36" s="22"/>
+      <x:c r="F36" s="22"/>
+      <x:c r="G36" s="22"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="C37" s="22"/>
+      <x:c r="D37" s="22"/>
+      <x:c r="E37" s="22"/>
+      <x:c r="F37" s="22"/>
+      <x:c r="G37" s="22"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="C38" s="22"/>
+      <x:c r="D38" s="22"/>
+      <x:c r="E38" s="22"/>
+      <x:c r="F38" s="22"/>
+      <x:c r="G38" s="22"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="C39" s="22"/>
+      <x:c r="D39" s="22"/>
+      <x:c r="E39" s="22"/>
+      <x:c r="F39" s="22"/>
+      <x:c r="G39" s="22"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="C40" s="22"/>
+      <x:c r="D40" s="22"/>
+      <x:c r="E40" s="22"/>
+      <x:c r="F40" s="22"/>
+      <x:c r="G40" s="22"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="C41" s="22"/>
+      <x:c r="D41" s="22"/>
+      <x:c r="E41" s="22"/>
+      <x:c r="F41" s="22"/>
+      <x:c r="G41" s="22"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="C42" s="22"/>
+      <x:c r="D42" s="22"/>
+      <x:c r="E42" s="22"/>
+      <x:c r="F42" s="22"/>
+      <x:c r="G42" s="22"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="C43" s="22"/>
+      <x:c r="D43" s="22"/>
+      <x:c r="E43" s="22"/>
+      <x:c r="F43" s="22"/>
+      <x:c r="G43" s="22"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="C44" s="22"/>
+      <x:c r="D44" s="22"/>
+      <x:c r="E44" s="22"/>
+      <x:c r="F44" s="22"/>
+      <x:c r="G44" s="22"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="C45" s="22"/>
+      <x:c r="D45" s="22"/>
+      <x:c r="E45" s="22"/>
+      <x:c r="F45" s="22"/>
+      <x:c r="G45" s="22"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="C46" s="22"/>
+      <x:c r="D46" s="22"/>
+      <x:c r="E46" s="22"/>
+      <x:c r="F46" s="22"/>
+      <x:c r="G46" s="22"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="C47" s="22"/>
+      <x:c r="D47" s="22"/>
+      <x:c r="E47" s="22"/>
+      <x:c r="F47" s="22"/>
+      <x:c r="G47" s="22"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="C48" s="22"/>
+      <x:c r="D48" s="22"/>
+      <x:c r="E48" s="22"/>
+      <x:c r="F48" s="22"/>
+      <x:c r="G48" s="22"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="C49" s="22"/>
+      <x:c r="D49" s="22"/>
+      <x:c r="E49" s="22"/>
+      <x:c r="F49" s="22"/>
+      <x:c r="G49" s="22"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="C50" s="22"/>
+      <x:c r="D50" s="22"/>
+      <x:c r="E50" s="22"/>
+      <x:c r="F50" s="22"/>
+      <x:c r="G50" s="22"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="C51" s="22"/>
+      <x:c r="D51" s="22"/>
+      <x:c r="E51" s="22"/>
+      <x:c r="F51" s="22"/>
+      <x:c r="G51" s="22"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="C52" s="22"/>
+      <x:c r="D52" s="22"/>
+      <x:c r="E52" s="22"/>
+      <x:c r="F52" s="22"/>
+      <x:c r="G52" s="22"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="C53" s="22"/>
+      <x:c r="D53" s="22"/>
+      <x:c r="E53" s="22"/>
+      <x:c r="F53" s="22"/>
+      <x:c r="G53" s="22"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="C54" s="22"/>
+      <x:c r="D54" s="22"/>
+      <x:c r="E54" s="22"/>
+      <x:c r="F54" s="22"/>
+      <x:c r="G54" s="22"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="C55" s="22"/>
+      <x:c r="D55" s="22"/>
+      <x:c r="E55" s="22"/>
+      <x:c r="F55" s="22"/>
+      <x:c r="G55" s="22"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="C56" s="22"/>
+      <x:c r="D56" s="22"/>
+      <x:c r="E56" s="22"/>
+      <x:c r="F56" s="22"/>
+      <x:c r="G56" s="22"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="C57" s="22"/>
+      <x:c r="D57" s="22"/>
+      <x:c r="E57" s="22"/>
+      <x:c r="F57" s="22"/>
+      <x:c r="G57" s="22"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="C58" s="22"/>
+      <x:c r="D58" s="22"/>
+      <x:c r="E58" s="22"/>
+      <x:c r="F58" s="22"/>
+      <x:c r="G58" s="22"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="C59" s="22"/>
+      <x:c r="D59" s="22"/>
+      <x:c r="E59" s="22"/>
+      <x:c r="F59" s="22"/>
+      <x:c r="G59" s="22"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="C60" s="22"/>
+      <x:c r="D60" s="22"/>
+      <x:c r="E60" s="22"/>
+      <x:c r="F60" s="22"/>
+      <x:c r="G60" s="22"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="C61" s="22"/>
+      <x:c r="D61" s="22"/>
+      <x:c r="E61" s="22"/>
+      <x:c r="F61" s="22"/>
+      <x:c r="G61" s="22"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="C62" s="22"/>
+      <x:c r="D62" s="22"/>
+      <x:c r="E62" s="22"/>
+      <x:c r="F62" s="22"/>
+      <x:c r="G62" s="22"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="C63" s="22"/>
+      <x:c r="D63" s="22"/>
+      <x:c r="E63" s="22"/>
+      <x:c r="F63" s="22"/>
+      <x:c r="G63" s="22"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="C64" s="22"/>
+      <x:c r="D64" s="22"/>
+      <x:c r="E64" s="22"/>
+      <x:c r="F64" s="22"/>
+      <x:c r="G64" s="22"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="C65" s="22"/>
+      <x:c r="D65" s="22"/>
+      <x:c r="E65" s="22"/>
+      <x:c r="F65" s="22"/>
+      <x:c r="G65" s="22"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="C66" s="22"/>
+      <x:c r="D66" s="22"/>
+      <x:c r="E66" s="22"/>
+      <x:c r="F66" s="22"/>
+      <x:c r="G66" s="22"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="C67" s="22"/>
+      <x:c r="D67" s="22"/>
+      <x:c r="E67" s="22"/>
+      <x:c r="F67" s="22"/>
+      <x:c r="G67" s="22"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="C68" s="22"/>
+      <x:c r="D68" s="22"/>
+      <x:c r="E68" s="22"/>
+      <x:c r="F68" s="22"/>
+      <x:c r="G68" s="22"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="C69" s="22"/>
+      <x:c r="D69" s="22"/>
+      <x:c r="E69" s="22"/>
+      <x:c r="F69" s="22"/>
+      <x:c r="G69" s="22"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="C70" s="22"/>
+      <x:c r="D70" s="22"/>
+      <x:c r="E70" s="22"/>
+      <x:c r="F70" s="22"/>
+      <x:c r="G70" s="22"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="C71" s="22"/>
+      <x:c r="D71" s="22"/>
+      <x:c r="E71" s="22"/>
+      <x:c r="F71" s="22"/>
+      <x:c r="G71" s="22"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="C72" s="22"/>
+      <x:c r="D72" s="22"/>
+      <x:c r="E72" s="22"/>
+      <x:c r="F72" s="22"/>
+      <x:c r="G72" s="22"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="C73" s="22"/>
+      <x:c r="D73" s="22"/>
+      <x:c r="E73" s="22"/>
+      <x:c r="F73" s="22"/>
+      <x:c r="G73" s="22"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="C74" s="22"/>
+      <x:c r="D74" s="22"/>
+      <x:c r="E74" s="22"/>
+      <x:c r="F74" s="22"/>
+      <x:c r="G74" s="22"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="C75" s="22"/>
+      <x:c r="D75" s="22"/>
+      <x:c r="E75" s="22"/>
+      <x:c r="F75" s="22"/>
+      <x:c r="G75" s="22"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="C76" s="22"/>
+      <x:c r="D76" s="22"/>
+      <x:c r="E76" s="22"/>
+      <x:c r="F76" s="22"/>
+      <x:c r="G76" s="22"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="C77" s="22"/>
+      <x:c r="D77" s="22"/>
+      <x:c r="E77" s="22"/>
+      <x:c r="F77" s="22"/>
+      <x:c r="G77" s="22"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="C78" s="22"/>
+      <x:c r="D78" s="22"/>
+      <x:c r="E78" s="22"/>
+      <x:c r="F78" s="22"/>
+      <x:c r="G78" s="22"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="C79" s="22"/>
+      <x:c r="D79" s="22"/>
+      <x:c r="E79" s="22"/>
+      <x:c r="F79" s="22"/>
+      <x:c r="G79" s="22"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="C80" s="22"/>
+      <x:c r="D80" s="22"/>
+      <x:c r="E80" s="22"/>
+      <x:c r="F80" s="22"/>
+      <x:c r="G80" s="22"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="C81" s="22"/>
+      <x:c r="D81" s="22"/>
+      <x:c r="E81" s="22"/>
+      <x:c r="F81" s="22"/>
+      <x:c r="G81" s="22"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="C82" s="22"/>
+      <x:c r="D82" s="22"/>
+      <x:c r="E82" s="22"/>
+      <x:c r="F82" s="22"/>
+      <x:c r="G82" s="22"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="C83" s="22"/>
+      <x:c r="D83" s="22"/>
+      <x:c r="E83" s="22"/>
+      <x:c r="F83" s="22"/>
+      <x:c r="G83" s="22"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="C84" s="22"/>
+      <x:c r="D84" s="22"/>
+      <x:c r="E84" s="22"/>
+      <x:c r="F84" s="22"/>
+      <x:c r="G84" s="22"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="C85" s="22"/>
+      <x:c r="D85" s="22"/>
+      <x:c r="E85" s="22"/>
+      <x:c r="F85" s="22"/>
+      <x:c r="G85" s="22"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="C86" s="22"/>
+      <x:c r="D86" s="22"/>
+      <x:c r="E86" s="22"/>
+      <x:c r="F86" s="22"/>
+      <x:c r="G86" s="22"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="C87" s="22"/>
+      <x:c r="D87" s="22"/>
+      <x:c r="E87" s="22"/>
+      <x:c r="F87" s="22"/>
+      <x:c r="G87" s="22"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="C88" s="22"/>
+      <x:c r="D88" s="22"/>
+      <x:c r="E88" s="22"/>
+      <x:c r="F88" s="22"/>
+      <x:c r="G88" s="22"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="C89" s="22"/>
+      <x:c r="D89" s="22"/>
+      <x:c r="E89" s="22"/>
+      <x:c r="F89" s="22"/>
+      <x:c r="G89" s="22"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="C90" s="22"/>
+      <x:c r="D90" s="22"/>
+      <x:c r="E90" s="22"/>
+      <x:c r="F90" s="22"/>
+      <x:c r="G90" s="22"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="C91" s="22"/>
+      <x:c r="D91" s="22"/>
+      <x:c r="E91" s="22"/>
+      <x:c r="F91" s="22"/>
+      <x:c r="G91" s="22"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="C92" s="22"/>
+      <x:c r="D92" s="22"/>
+      <x:c r="E92" s="22"/>
+      <x:c r="F92" s="22"/>
+      <x:c r="G92" s="22"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="C93" s="22"/>
+      <x:c r="D93" s="22"/>
+      <x:c r="E93" s="22"/>
+      <x:c r="F93" s="22"/>
+      <x:c r="G93" s="22"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="C94" s="22"/>
+      <x:c r="D94" s="22"/>
+      <x:c r="E94" s="22"/>
+      <x:c r="F94" s="22"/>
+      <x:c r="G94" s="22"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="C95" s="22"/>
+      <x:c r="D95" s="22"/>
+      <x:c r="E95" s="22"/>
+      <x:c r="F95" s="22"/>
+      <x:c r="G95" s="22"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="C96" s="22"/>
+      <x:c r="D96" s="22"/>
+      <x:c r="E96" s="22"/>
+      <x:c r="F96" s="22"/>
+      <x:c r="G96" s="22"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="C97" s="22"/>
+      <x:c r="D97" s="22"/>
+      <x:c r="E97" s="22"/>
+      <x:c r="F97" s="22"/>
+      <x:c r="G97" s="22"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="C98" s="22"/>
+      <x:c r="D98" s="22"/>
+      <x:c r="E98" s="22"/>
+      <x:c r="F98" s="22"/>
+      <x:c r="G98" s="22"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="C99" s="22"/>
+      <x:c r="D99" s="22"/>
+      <x:c r="E99" s="22"/>
+      <x:c r="F99" s="22"/>
+      <x:c r="G99" s="22"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="C100" s="22"/>
+      <x:c r="D100" s="22"/>
+      <x:c r="E100" s="22"/>
+      <x:c r="F100" s="22"/>
+      <x:c r="G100" s="22"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -838,6 +1727,7 @@
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -852,6 +1742,7 @@
       <x:c r="G1" s="4"/>
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
@@ -881,6 +1772,9 @@
       <x:c r="I3" s="10" t="str">
         <x:v>Source Mode</x:v>
       </x:c>
+      <x:c r="J3" s="10" t="str">
+        <x:v>Note</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -889,19 +1783,19 @@
       <x:c r="B4" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C4" s="20" t="n">
+      <x:c r="C4" s="26" t="n">
         <x:v>0.82</x:v>
       </x:c>
-      <x:c r="D4" s="20" t="n">
+      <x:c r="D4" s="26" t="n">
         <x:v>0.36</x:v>
       </x:c>
-      <x:c r="E4" s="20" t="n">
+      <x:c r="E4" s="26" t="n">
         <x:v>0.015</x:v>
       </x:c>
-      <x:c r="F4" s="20" t="n">
+      <x:c r="F4" s="26" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G4" s="20" t="n">
+      <x:c r="G4" s="26" t="n">
         <x:v>0.034</x:v>
       </x:c>
       <x:c r="H4" t="str">
@@ -909,6 +1803,9 @@
       </x:c>
       <x:c r="I4" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -918,19 +1815,19 @@
       <x:c r="B5" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C5" s="20" t="n">
+      <x:c r="C5" s="26" t="n">
         <x:v>0.88</x:v>
       </x:c>
-      <x:c r="D5" s="20" t="n">
+      <x:c r="D5" s="26" t="n">
         <x:v>0.18</x:v>
       </x:c>
-      <x:c r="E5" s="20" t="n">
+      <x:c r="E5" s="26" t="n">
         <x:v>0.035</x:v>
       </x:c>
-      <x:c r="F5" s="20" t="n">
+      <x:c r="F5" s="26" t="n">
         <x:v>0.05</x:v>
       </x:c>
-      <x:c r="G5" s="20" t="n">
+      <x:c r="G5" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="H5" t="str">
@@ -938,6 +1835,9 @@
       </x:c>
       <x:c r="I5" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -947,19 +1847,19 @@
       <x:c r="B6" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C6" s="20" t="n">
+      <x:c r="C6" s="26" t="n">
         <x:v>0.87</x:v>
       </x:c>
-      <x:c r="D6" s="20" t="n">
+      <x:c r="D6" s="26" t="n">
         <x:v>0.22</x:v>
       </x:c>
-      <x:c r="E6" s="20" t="n">
+      <x:c r="E6" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="F6" s="20" t="n">
+      <x:c r="F6" s="26" t="n">
         <x:v>0.04</x:v>
       </x:c>
-      <x:c r="G6" s="20" t="n">
+      <x:c r="G6" s="26" t="n">
         <x:v>0.031</x:v>
       </x:c>
       <x:c r="H6" t="str">
@@ -967,6 +1867,9 @@
       </x:c>
       <x:c r="I6" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -976,19 +1879,19 @@
       <x:c r="B7" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C7" s="20" t="n">
+      <x:c r="C7" s="26" t="n">
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="D7" s="20" t="n">
+      <x:c r="D7" s="26" t="n">
         <x:v>0.38</x:v>
       </x:c>
-      <x:c r="E7" s="20" t="n">
+      <x:c r="E7" s="26" t="n">
         <x:v>0.01</x:v>
       </x:c>
-      <x:c r="F7" s="20" t="n">
+      <x:c r="F7" s="26" t="n">
         <x:v>-0.02</x:v>
       </x:c>
-      <x:c r="G7" s="20" t="n">
+      <x:c r="G7" s="26" t="n">
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="H7" t="str">
@@ -996,6 +1899,9 @@
       </x:c>
       <x:c r="I7" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1005,19 +1911,19 @@
       <x:c r="B8" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C8" s="20" t="n">
+      <x:c r="C8" s="26" t="n">
         <x:v>0.83</x:v>
       </x:c>
-      <x:c r="D8" s="20" t="n">
+      <x:c r="D8" s="26" t="n">
         <x:v>0.4</x:v>
       </x:c>
-      <x:c r="E8" s="20" t="n">
+      <x:c r="E8" s="26" t="n">
         <x:v>0.02</x:v>
       </x:c>
-      <x:c r="F8" s="20" t="n">
+      <x:c r="F8" s="26" t="n">
         <x:v>0.01</x:v>
       </x:c>
-      <x:c r="G8" s="20" t="n">
+      <x:c r="G8" s="26" t="n">
         <x:v>0.041</x:v>
       </x:c>
       <x:c r="H8" t="str">
@@ -1025,6 +1931,9 @@
       </x:c>
       <x:c r="I8" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1034,19 +1943,19 @@
       <x:c r="B9" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C9" s="20" t="n">
+      <x:c r="C9" s="26" t="n">
         <x:v>0.84</x:v>
       </x:c>
-      <x:c r="D9" s="20" t="n">
+      <x:c r="D9" s="26" t="n">
         <x:v>0.23</x:v>
       </x:c>
-      <x:c r="E9" s="20" t="n">
+      <x:c r="E9" s="26" t="n">
         <x:v>0.015</x:v>
       </x:c>
-      <x:c r="F9" s="20" t="n">
+      <x:c r="F9" s="26" t="n">
         <x:v>0.02</x:v>
       </x:c>
-      <x:c r="G9" s="20" t="n">
+      <x:c r="G9" s="26" t="n">
         <x:v>0.037</x:v>
       </x:c>
       <x:c r="H9" t="str">
@@ -1054,6 +1963,9 @@
       </x:c>
       <x:c r="I9" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1063,19 +1975,19 @@
       <x:c r="B10" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C10" s="20" t="n">
+      <x:c r="C10" s="26" t="n">
         <x:v>0.88</x:v>
       </x:c>
-      <x:c r="D10" s="20" t="n">
+      <x:c r="D10" s="26" t="n">
         <x:v>0.19</x:v>
       </x:c>
-      <x:c r="E10" s="20" t="n">
+      <x:c r="E10" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="F10" s="20" t="n">
+      <x:c r="F10" s="26" t="n">
         <x:v>0.07</x:v>
       </x:c>
-      <x:c r="G10" s="20" t="n">
+      <x:c r="G10" s="26" t="n">
         <x:v>0.045</x:v>
       </x:c>
       <x:c r="H10" t="str">
@@ -1083,6 +1995,9 @@
       </x:c>
       <x:c r="I10" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1092,19 +2007,19 @@
       <x:c r="B11" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C11" s="20" t="n">
+      <x:c r="C11" s="26" t="n">
         <x:v>0.91</x:v>
       </x:c>
-      <x:c r="D11" s="20" t="n">
+      <x:c r="D11" s="26" t="n">
         <x:v>0.16</x:v>
       </x:c>
-      <x:c r="E11" s="20" t="n">
+      <x:c r="E11" s="26" t="n">
         <x:v>0.045</x:v>
       </x:c>
-      <x:c r="F11" s="20" t="n">
+      <x:c r="F11" s="26" t="n">
         <x:v>0.09</x:v>
       </x:c>
-      <x:c r="G11" s="20" t="n">
+      <x:c r="G11" s="26" t="n">
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="H11" t="str">
@@ -1112,6 +2027,9 @@
       </x:c>
       <x:c r="I11" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1121,19 +2039,19 @@
       <x:c r="B12" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C12" s="20" t="n">
+      <x:c r="C12" s="26" t="n">
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="D12" s="20" t="n">
+      <x:c r="D12" s="26" t="n">
         <x:v>0.18</x:v>
       </x:c>
-      <x:c r="E12" s="20" t="n">
+      <x:c r="E12" s="26" t="n">
         <x:v>0.025</x:v>
       </x:c>
-      <x:c r="F12" s="20" t="n">
+      <x:c r="F12" s="26" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="G12" s="20" t="n">
+      <x:c r="G12" s="26" t="n">
         <x:v>0.035</x:v>
       </x:c>
       <x:c r="H12" t="str">
@@ -1141,6 +2059,9 @@
       </x:c>
       <x:c r="I12" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1150,19 +2071,19 @@
       <x:c r="B13" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C13" s="20" t="n">
+      <x:c r="C13" s="26" t="n">
         <x:v>0.92</x:v>
       </x:c>
-      <x:c r="D13" s="20" t="n">
+      <x:c r="D13" s="26" t="n">
         <x:v>0.17</x:v>
       </x:c>
-      <x:c r="E13" s="20" t="n">
+      <x:c r="E13" s="26" t="n">
         <x:v>0.035</x:v>
       </x:c>
-      <x:c r="F13" s="20" t="n">
+      <x:c r="F13" s="26" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="G13" s="20" t="n">
+      <x:c r="G13" s="26" t="n">
         <x:v>0.043</x:v>
       </x:c>
       <x:c r="H13" t="str">
@@ -1170,6 +2091,9 @@
       </x:c>
       <x:c r="I13" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1179,19 +2103,19 @@
       <x:c r="B14" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C14" s="20" t="n">
+      <x:c r="C14" s="26" t="n">
         <x:v>0.89</x:v>
       </x:c>
-      <x:c r="D14" s="20" t="n">
+      <x:c r="D14" s="26" t="n">
         <x:v>0.14</x:v>
       </x:c>
-      <x:c r="E14" s="20" t="n">
+      <x:c r="E14" s="26" t="n">
         <x:v>0.04</x:v>
       </x:c>
-      <x:c r="F14" s="20" t="n">
+      <x:c r="F14" s="26" t="n">
         <x:v>0.07</x:v>
       </x:c>
-      <x:c r="G14" s="20" t="n">
+      <x:c r="G14" s="26" t="n">
         <x:v>0.032</x:v>
       </x:c>
       <x:c r="H14" t="str">
@@ -1199,6 +2123,9 @@
       </x:c>
       <x:c r="I14" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1208,19 +2135,19 @@
       <x:c r="B15" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C15" s="20" t="n">
+      <x:c r="C15" s="26" t="n">
         <x:v>0.87</x:v>
       </x:c>
-      <x:c r="D15" s="20" t="n">
+      <x:c r="D15" s="26" t="n">
         <x:v>0.23</x:v>
       </x:c>
-      <x:c r="E15" s="20" t="n">
+      <x:c r="E15" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="F15" s="20" t="n">
+      <x:c r="F15" s="26" t="n">
         <x:v>0.05</x:v>
       </x:c>
-      <x:c r="G15" s="20" t="n">
+      <x:c r="G15" s="26" t="n">
         <x:v>0.038</x:v>
       </x:c>
       <x:c r="H15" t="str">
@@ -1228,6 +2155,9 @@
       </x:c>
       <x:c r="I15" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1237,19 +2167,19 @@
       <x:c r="B16" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C16" s="20" t="n">
+      <x:c r="C16" s="26" t="n">
         <x:v>0.86</x:v>
       </x:c>
-      <x:c r="D16" s="20" t="n">
+      <x:c r="D16" s="26" t="n">
         <x:v>0.13</x:v>
       </x:c>
-      <x:c r="E16" s="20" t="n">
+      <x:c r="E16" s="26" t="n">
         <x:v>0.025</x:v>
       </x:c>
-      <x:c r="F16" s="20" t="n">
+      <x:c r="F16" s="26" t="n">
         <x:v>0.04</x:v>
       </x:c>
-      <x:c r="G16" s="20" t="n">
+      <x:c r="G16" s="26" t="n">
         <x:v>0.036</x:v>
       </x:c>
       <x:c r="H16" t="str">
@@ -1257,6 +2187,9 @@
       </x:c>
       <x:c r="I16" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1266,19 +2199,19 @@
       <x:c r="B17" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C17" s="20" t="n">
+      <x:c r="C17" s="26" t="n">
         <x:v>0.91</x:v>
       </x:c>
-      <x:c r="D17" s="20" t="n">
+      <x:c r="D17" s="26" t="n">
         <x:v>0.15</x:v>
       </x:c>
-      <x:c r="E17" s="20" t="n">
+      <x:c r="E17" s="26" t="n">
         <x:v>0.035</x:v>
       </x:c>
-      <x:c r="F17" s="20" t="n">
+      <x:c r="F17" s="26" t="n">
         <x:v>0.09</x:v>
       </x:c>
-      <x:c r="G17" s="20" t="n">
+      <x:c r="G17" s="26" t="n">
         <x:v>0.034</x:v>
       </x:c>
       <x:c r="H17" t="str">
@@ -1286,6 +2219,9 @@
       </x:c>
       <x:c r="I17" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1295,19 +2231,19 @@
       <x:c r="B18" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C18" s="20" t="n">
+      <x:c r="C18" s="26" t="n">
         <x:v>0.82</x:v>
       </x:c>
-      <x:c r="D18" s="20" t="n">
+      <x:c r="D18" s="26" t="n">
         <x:v>0.27</x:v>
       </x:c>
-      <x:c r="E18" s="20" t="n">
+      <x:c r="E18" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="F18" s="20" t="n">
+      <x:c r="F18" s="26" t="n">
         <x:v>0.01</x:v>
       </x:c>
-      <x:c r="G18" s="20" t="n">
+      <x:c r="G18" s="26" t="n">
         <x:v>0.038</x:v>
       </x:c>
       <x:c r="H18" t="str">
@@ -1315,6 +2251,9 @@
       </x:c>
       <x:c r="I18" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1324,19 +2263,19 @@
       <x:c r="B19" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C19" s="20" t="n">
+      <x:c r="C19" s="26" t="n">
         <x:v>0.79</x:v>
       </x:c>
-      <x:c r="D19" s="20" t="n">
+      <x:c r="D19" s="26" t="n">
         <x:v>0.12</x:v>
       </x:c>
-      <x:c r="E19" s="20" t="n">
+      <x:c r="E19" s="26" t="n">
         <x:v>0.025</x:v>
       </x:c>
-      <x:c r="F19" s="20" t="n">
+      <x:c r="F19" s="26" t="n">
         <x:v>-0.03</x:v>
       </x:c>
-      <x:c r="G19" s="20" t="n">
+      <x:c r="G19" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="H19" t="str">
@@ -1344,6 +2283,9 @@
       </x:c>
       <x:c r="I19" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1353,19 +2295,19 @@
       <x:c r="B20" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C20" s="20" t="n">
+      <x:c r="C20" s="26" t="n">
         <x:v>0.77</x:v>
       </x:c>
-      <x:c r="D20" s="20" t="n">
+      <x:c r="D20" s="26" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="E20" s="20" t="n">
+      <x:c r="E20" s="26" t="n">
         <x:v>0.02</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="n">
+      <x:c r="F20" s="26" t="n">
         <x:v>-0.05</x:v>
       </x:c>
-      <x:c r="G20" s="20" t="n">
+      <x:c r="G20" s="26" t="n">
         <x:v>0.028</x:v>
       </x:c>
       <x:c r="H20" t="str">
@@ -1373,6 +2315,9 @@
       </x:c>
       <x:c r="I20" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1382,19 +2327,19 @@
       <x:c r="B21" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C21" s="20" t="n">
+      <x:c r="C21" s="26" t="n">
         <x:v>0.88</x:v>
       </x:c>
-      <x:c r="D21" s="20" t="n">
+      <x:c r="D21" s="26" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="E21" s="20" t="n">
+      <x:c r="E21" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="F21" s="20" t="n">
+      <x:c r="F21" s="26" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="G21" s="20" t="n">
+      <x:c r="G21" s="26" t="n">
         <x:v>0.033</x:v>
       </x:c>
       <x:c r="H21" t="str">
@@ -1402,6 +2347,9 @@
       </x:c>
       <x:c r="I21" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1411,19 +2359,19 @@
       <x:c r="B22" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C22" s="20" t="n">
+      <x:c r="C22" s="26" t="n">
         <x:v>0.84</x:v>
       </x:c>
-      <x:c r="D22" s="20" t="n">
+      <x:c r="D22" s="26" t="n">
         <x:v>0.09</x:v>
       </x:c>
-      <x:c r="E22" s="20" t="n">
+      <x:c r="E22" s="26" t="n">
         <x:v>0.025</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="n">
+      <x:c r="F22" s="26" t="n">
         <x:v>0.04</x:v>
       </x:c>
-      <x:c r="G22" s="20" t="n">
+      <x:c r="G22" s="26" t="n">
         <x:v>0.034</x:v>
       </x:c>
       <x:c r="H22" t="str">
@@ -1431,6 +2379,9 @@
       </x:c>
       <x:c r="I22" t="str">
         <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1440,19 +2391,19 @@
       <x:c r="B23" t="str">
         <x:v>Fallback</x:v>
       </x:c>
-      <x:c r="C23" s="20" t="n">
+      <x:c r="C23" s="26" t="n">
         <x:v>0.83</x:v>
       </x:c>
-      <x:c r="D23" s="20" t="n">
+      <x:c r="D23" s="26" t="n">
         <x:v>0.07</x:v>
       </x:c>
-      <x:c r="E23" s="20" t="n">
+      <x:c r="E23" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="F23" s="20" t="n">
+      <x:c r="F23" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
-      <x:c r="G23" s="20" t="n">
+      <x:c r="G23" s="26" t="n">
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="H23" t="str">
@@ -1461,16 +2412,19 @@
       <x:c r="I23" t="str">
         <x:v>FALLBACK</x:v>
       </x:c>
+      <x:c r="J23" t="str">
+        <x:v>Chỉ dùng khi Bronze ACTUAL thiếu</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1480,15 +2434,15 @@
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>SPONSOR CONNECTION CONTROL PANEL</x:v>
+        <x:v>PRODUCTION CONTROL PANEL</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1513,19 +2467,19 @@
       <x:c r="D3" s="10" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F3" s="22" t="str">
-        <x:v>CONNECTION UX</x:v>
-      </x:c>
-      <x:c r="G3" s="22"/>
-      <x:c r="H3" s="22"/>
-      <x:c r="I3" s="22"/>
-      <x:c r="J3" s="22"/>
+      <x:c r="F3" s="28" t="str">
+        <x:v>PRODUCTION GUARANTEES</x:v>
+      </x:c>
+      <x:c r="G3" s="28"/>
+      <x:c r="H3" s="28"/>
+      <x:c r="I3" s="28"/>
+      <x:c r="J3" s="28"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
         <x:v>Credit growth YTD</x:v>
       </x:c>
-      <x:c r="B4" t="n">
+      <x:c r="B4" s="16" t="n">
         <x:v>7.41</x:v>
       </x:c>
       <x:c r="C4" t="str">
@@ -1535,26 +2489,22 @@
         <x:v>ACTUAL</x:v>
       </x:c>
       <x:c r="F4" s="10" t="str">
-        <x:v>State</x:v>
+        <x:v>Rule</x:v>
       </x:c>
       <x:c r="G4" s="10" t="str">
-        <x:v>Button visible?</x:v>
+        <x:v>Setting</x:v>
       </x:c>
       <x:c r="H4" s="10" t="str">
-        <x:v>Action</x:v>
-      </x:c>
-      <x:c r="I4" s="10" t="str">
-        <x:v>Expected result</x:v>
-      </x:c>
-      <x:c r="J4" s="10" t="str">
-        <x:v>Fallback</x:v>
-      </x:c>
+        <x:v>Why</x:v>
+      </x:c>
+      <x:c r="I4" t="str"/>
+      <x:c r="J4" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
         <x:v>Deposit growth YTD</x:v>
       </x:c>
-      <x:c r="B5" t="n">
+      <x:c r="B5" s="16" t="n">
         <x:v>5.02</x:v>
       </x:c>
       <x:c r="C5" t="str">
@@ -1564,26 +2514,22 @@
         <x:v>ACTUAL</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>No API Key</x:v>
+        <x:v>Sponsor environment</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>No</x:v>
+        <x:v>Persistent PC/server</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>Enter key</x:v>
-      </x:c>
-      <x:c r="I5" t="str">
-        <x:v>Key configured</x:v>
-      </x:c>
-      <x:c r="J5" t="str">
-        <x:v>Free</x:v>
-      </x:c>
+        <x:v>Avoid ephemeral device activation</x:v>
+      </x:c>
+      <x:c r="I5" t="str"/>
+      <x:c r="J5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
         <x:v>Funding gap</x:v>
       </x:c>
-      <x:c r="B6" t="n">
+      <x:c r="B6" s="16" t="n">
         <x:f>B4-B5</x:f>
         <x:v>2.3900000000000006</x:v>
       </x:c>
@@ -1594,26 +2540,22 @@
         <x:v>CALC</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Key + no Sponsor</x:v>
+        <x:v>Streamlit API calls</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>YES</x:v>
+        <x:v>Zero</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>Connect Bronze</x:v>
-      </x:c>
-      <x:c r="I6" t="str">
-        <x:v>Install/activate vnstock_data</x:v>
-      </x:c>
-      <x:c r="J6" t="str">
-        <x:v>Free</x:v>
-      </x:c>
+        <x:v>No rate-limit / installer failure</x:v>
+      </x:c>
+      <x:c r="I6" t="str"/>
+      <x:c r="J6" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
         <x:v>CPI YoY</x:v>
       </x:c>
-      <x:c r="B7" t="n">
+      <x:c r="B7" s="16" t="n">
         <x:v>4.69</x:v>
       </x:c>
       <x:c r="C7" t="str">
@@ -1623,26 +2565,22 @@
         <x:v>ACTUAL</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Sponsor connected</x:v>
+        <x:v>Actual source</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>No</x:v>
+        <x:v>Bronze CSV</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>Auto data probe</x:v>
-      </x:c>
-      <x:c r="I7" t="str">
-        <x:v>Bronze ACTUAL</x:v>
-      </x:c>
-      <x:c r="J7" t="str">
-        <x:v>Free</x:v>
-      </x:c>
+        <x:v>Traceable actual data</x:v>
+      </x:c>
+      <x:c r="I7" t="str"/>
+      <x:c r="J7" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
         <x:v>Trade balance 6M</x:v>
       </x:c>
-      <x:c r="B8" t="n">
+      <x:c r="B8" s="16" t="n">
         <x:v>-16.65</x:v>
       </x:c>
       <x:c r="C8" t="str">
@@ -1652,48 +2590,54 @@
         <x:v>ACTUAL</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>Bronze probe fail</x:v>
+        <x:v>Automation</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>No</x:v>
+        <x:v>Self-hosted runner</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>Circuit opens</x:v>
-      </x:c>
-      <x:c r="I8" t="str">
-        <x:v>No repeated calls</x:v>
-      </x:c>
-      <x:c r="J8" t="str">
-        <x:v>Free</x:v>
-      </x:c>
+        <x:v>Stable scheduled refresh</x:v>
+      </x:c>
+      <x:c r="I8" t="str"/>
+      <x:c r="J8" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Free full-universe calls</x:v>
-      </x:c>
-      <x:c r="B9" t="n">
+        <x:v>Streamlit Vnstock calls</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>banks</x:v>
+        <x:v>requests</x:v>
       </x:c>
       <x:c r="D9" t="str">
         <x:v>CONTROL</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>Free probe fail</x:v>
+        <x:v>Fallback</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>No</x:v>
+        <x:v>Explicit assumption</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>Circuit opens</x:v>
-      </x:c>
-      <x:c r="I9" t="str">
-        <x:v>Fallback</x:v>
-      </x:c>
-      <x:c r="J9" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Dashboard remains usable</x:v>
+      </x:c>
+      <x:c r="I9" t="str"/>
+      <x:c r="J9" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Streamlit Sponsor installer</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>runs</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>CONTROL</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Refine LPI interbank and bank stress models
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9d57c28954a24af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARCHITECTURE" sheetId="2" r:id="R1cce0a67aa2a4573"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_STACK" sheetId="3" r:id="R157b8b41347d4c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LPI_METHOD" sheetId="4" r:id="Reb3a527c4f7c40ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORECAST_CONFIG" sheetId="5" r:id="Rc495fb9d811d4f81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_DIAGNOSTICS" sheetId="6" r:id="Rb2f991c0bec64426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_STRESS" sheetId="7" r:id="R55e15a4fdbb149fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCENARIOS" sheetId="8" r:id="Rb48979d87edd47bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA_LINEAGE" sheetId="9" r:id="R1d701fafe6b24816"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="10" r:id="R71b87ce7ed3042b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R16b83e6865154add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARCHITECTURE" sheetId="2" r:id="Rbfaf9e4244ae4375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_STACK" sheetId="3" r:id="R810748f316fd4e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LPI_METHOD" sheetId="4" r:id="R4a334f96a4f94f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORECAST_CONFIG" sheetId="5" r:id="R24229f1e09f64307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_DIAGNOSTICS" sheetId="6" r:id="Re936efa665bb486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_STRESS" sheetId="7" r:id="Ra6e7ca684b8e4140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCENARIOS" sheetId="8" r:id="R2f7af49684e047ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA_LINEAGE" sheetId="9" r:id="R1de1203dbc3b4750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="10" r:id="R5652bf4660544240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFINEMENTS" sheetId="11" r:id="Rf59dfd3fa43c4cc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,6 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="0%"/>
+    <x:numFmt numFmtId="201" formatCode="0.00"/>
+  </x:numFmts>
   <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
@@ -45,12 +50,27 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2747"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -75,7 +95,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -110,6 +130,24 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -749,6 +787,424 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="29" t="str">
+        <x:v>UI &amp; MODEL REFINEMENTS</x:v>
+      </x:c>
+      <x:c r="B1" s="29"/>
+      <x:c r="C1" s="29"/>
+      <x:c r="D1" s="29"/>
+      <x:c r="E1" s="29"/>
+      <x:c r="F1" s="29"/>
+      <x:c r="G1" s="29"/>
+      <x:c r="H1" s="29"/>
+      <x:c r="I1" s="29"/>
+      <x:c r="J1" s="29"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="28" t="str">
+        <x:v>Issue</x:v>
+      </x:c>
+      <x:c r="B3" s="28" t="str">
+        <x:v>Observed symptom</x:v>
+      </x:c>
+      <x:c r="C3" s="28" t="str">
+        <x:v>Root cause</x:v>
+      </x:c>
+      <x:c r="D3" s="28" t="str">
+        <x:v>Fix</x:v>
+      </x:c>
+      <x:c r="E3" s="28" t="str">
+        <x:v>Data policy</x:v>
+      </x:c>
+      <x:c r="F3" s="28" t="str">
+        <x:v>Production behavior</x:v>
+      </x:c>
+      <x:c r="G3" s="28" t="str">
+        <x:v>User impact</x:v>
+      </x:c>
+      <x:c r="H3" s="28" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="I3" s="28" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="J3" s="28" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Top header</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Title partly clipped</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Insufficient top padding / line height</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Increase top padding; responsive title size</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>UI only</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Full title visible</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I4" t="str"/>
+      <x:c r="J4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>LPI chart</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Hard to interpret</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Too much history + forecast bands without thresholds</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>12-month forecast view + threshold bands + economic labels</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>No data change</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>Faster interpretation</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I5" t="str"/>
+      <x:c r="J5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>LPI drivers</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Too noisy</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Multi-year component chart</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>18-month focused driver chart; LPI emphasized</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>No data change</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Drivers easier to read</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I6" t="str"/>
+      <x:c r="J6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Regime chart</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Highly jagged</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Daily Markov probabilities</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>20-day smoothing for display; raw probabilities retained</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Raw model unchanged</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Regime trend clearer</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I7" t="str"/>
+      <x:c r="J7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Interbank</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>No chart/forecast</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Dedicated endpoint returned 404</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Fallback chain: interbank_rate → currency.interest_rate → legacy interest_rate</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Never synthesize rates</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Actual series appears if any official endpoint works</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>https://vnstocks.com/docs/vnstock-data/macro-layer-v3</x:v>
+      </x:c>
+      <x:c r="J8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Bank stress</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Blank bars</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Bronze rows labelled ACTUAL but quantitative metrics were null</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Use Bronze only at &gt;=60% metric coverage; otherwise ticker-level ASSUMPTION fallback</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>ACTUAL &gt; ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>No null vulnerability bars</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Stress chart populated</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I9" t="str"/>
+      <x:c r="J9" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Custom stress</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Blank bars</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>BaseVulnerability null</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Scenario engine filters valid base rows and uses ticker-level fallback</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>ASSUMPTION scenario</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Scenario sliders remain assumptions</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Stress Lab populated</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>FIXED</x:v>
+      </x:c>
+      <x:c r="I10" t="str"/>
+      <x:c r="J10" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="30" t="str">
+        <x:v>BANK STRESS DATA GATE</x:v>
+      </x:c>
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="27" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>Threshold</x:v>
+      </x:c>
+      <x:c r="C13" s="27" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="D13" s="27" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="E13" s="27" t="str">
+        <x:v>If pass</x:v>
+      </x:c>
+      <x:c r="F13" s="27" t="str">
+        <x:v>If fail</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="str">
+        <x:v>Rationale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Bronze metric coverage</x:v>
+      </x:c>
+      <x:c r="B14" s="32" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>At least 3/5 metrics available</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Use BRONZE ACTUAL</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Fallback ticker to ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Avoid blank/false precision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>Metrics</x:v>
+      </x:c>
+      <x:c r="B15" s="31" t="str">
+        <x:v>LDR/CASA/InterbankDep/CreditDepositGap/NIM</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Core funding variables</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>Calculate vulnerability</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Do not score actual row</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Transparent data gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>Stress threshold AMBER</x:v>
+      </x:c>
+      <x:c r="B16" s="31" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Monitoring zone</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>AMBER</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Below = GREEN</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Risk rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>Stress threshold RED</x:v>
+      </x:c>
+      <x:c r="B17" s="33" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>High stress zone</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>RED</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Below = AMBER/GREEN</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Risk rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>NIM red trigger</x:v>
+      </x:c>
+      <x:c r="B18" s="33" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Stressed NIM below 2%</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>RED</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Otherwise score threshold applies</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Profit-buffer rule</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A12:G12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
Upgrade liquidity intelligence Production R3
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra3b9e166c11645d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_GOVERNANCE" sheetId="2" r:id="R208af5d7a4a74077"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_STRESS" sheetId="3" r:id="Rfd0408a137174b82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_INPUT" sheetId="4" r:id="R1032c51eecc54bf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPGRADE_CHECKLIST" sheetId="5" r:id="R34c1cd0a1fd2461c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="6" r:id="Rdad72cfc5b9d49e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1d6761a806a94f44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRESS_FALLBACK" sheetId="2" r:id="R037099c50bfe4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORECAST_GOVERNANCE" sheetId="3" r:id="R7584c061d5704ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_INPUT" sheetId="4" r:id="Ra5b94073ea5a4ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R3_VALIDATION" sheetId="5" r:id="R85ea4db7cbad4735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPGRADE_CHECKLIST" sheetId="6" r:id="R96b503b0b2944950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DASHBOARD" sheetId="7" r:id="Re45c25b6f41a4987"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,8 +20,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="3">
-    <x:numFmt numFmtId="200" formatCode="0.00"/>
-    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
   </x:numFmts>
   <x:fonts count="4">
@@ -317,12 +318,12 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="100" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="105" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>VIETNAM BANKING LIQUIDITY INTELLIGENCE — PRODUCTION R2</x:v>
+        <x:v>VIETNAM BANKING LIQUIDITY INTELLIGENCE — PRODUCTION R3</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="4"/>
@@ -342,42 +343,42 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Bronze architecture</x:v>
+        <x:v>Kiến trúc</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Persistent PC/self-hosted → vnstock_data Bronze → ACTUAL CSV → model outputs → GitHub → Streamlit.</x:v>
+        <x:v>Persistent PC/self-hosted → vnstock_data Bronze → ACTUAL CSV → governed models → GitHub → Streamlit.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Cloud policy</x:v>
+        <x:v>Upgrade</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Streamlit không cài/gọi Vnstock Sponsor.</x:v>
+        <x:v>CODE ONLY; package không chứa data/. Giữ nguyên data/ production.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Upgrade policy</x:v>
+        <x:v>Stress guarantee</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Package CODE ONLY không chứa data/. Giữ nguyên data/ production khi nâng cấp.</x:v>
+        <x:v>2 lớp fallback: build_models + runtime app. Funding Stress/Stress Lab không được phép trống.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Forecast governance</x:v>
+        <x:v>Fallback labeling</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>ARIMA chỉ được công bố nếu RMSE holdout tốt hơn naive benchmark; nếu không dùng NAIVE_RANDOM_WALK, Confidence=LOW.</x:v>
+        <x:v>Mọi fallback ghi rõ ASSUMPTION / FALLBACK, không giả làm Bronze.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Bank stress</x:v>
+        <x:v>Forecast governance</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Bronze chỉ dùng khi &gt;=60% coverage; thiếu thì fallback riêng từng ticker với nhãn ASSUMPTION.</x:v>
+        <x:v>ARIMA chỉ dùng nếu RMSE holdout thấp hơn naive; nếu không dùng NAIVE_RANDOM_WALK, Confidence=LOW.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -385,30 +386,22 @@
         <x:v>Interbank</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Chỉ true interbank. Không dùng deposit/lending rate proxy để giả làm interbank.</x:v>
+        <x:v>Chỉ true interbank Bronze/manual ACTUAL; funding-rate proxy hiển thị riêng, không dùng forecast ON.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Manual interbank</x:v>
+        <x:v>Test</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>Có thể nhập ACTUAL vào sheet INTERBANK_INPUT; cần &gt;=10 dòng hợp lệ có source URL.</x:v>
+        <x:v>Đã mô phỏng 20 bank Bronze coverage=0: model sinh đủ 20 BaseVulnerability từ fallback.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>UI fixes</x:v>
+        <x:v>Refresh</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Không còn DeltaGenerator bị in ra; Diagnostics/Sidebar dùng if/else rõ ràng.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>Refresh</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
         <x:v>REFRESH_BRONZE_BUILD_MODELS_AND_PUSH.bat</x:v>
       </x:c>
     </x:row>
@@ -424,20 +417,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="44" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="46" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>FORECAST MODEL GOVERNANCE</x:v>
+        <x:v>BANK STRESS FALLBACK GOVERNANCE</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -450,205 +443,147 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>Rule</x:v>
+        <x:v>Layer</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
-        <x:v>Threshold / Method</x:v>
+        <x:v>Trigger</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
-        <x:v>Type</x:v>
+        <x:v>Action</x:v>
       </x:c>
       <x:c r="D3" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Output</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
-        <x:v>Pass condition</x:v>
+        <x:v>Data Type</x:v>
       </x:c>
       <x:c r="F3" s="10" t="str">
-        <x:v>Fail action</x:v>
+        <x:v>Source Mode</x:v>
       </x:c>
       <x:c r="G3" s="10" t="str">
-        <x:v>Output label</x:v>
+        <x:v>Can be blank?</x:v>
       </x:c>
       <x:c r="H3" s="10" t="str">
-        <x:v>Why</x:v>
+        <x:v>Control</x:v>
       </x:c>
       <x:c r="I3" s="10" t="str">
-        <x:v>User interpretation</x:v>
+        <x:v>Interpretation</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Minimum daily history</x:v>
-      </x:c>
-      <x:c r="B4" s="18" t="n">
-        <x:v>80</x:v>
+        <x:v>Model build</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Bronze coverage &gt;=60%</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>ASSUMPTION</x:v>
+        <x:v>Use Bronze quantitative metrics</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>LPI/Interbank</x:v>
+        <x:v>BaseVulnerability</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>&gt;=80 obs</x:v>
+        <x:v>ACTUAL</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>No forecast</x:v>
+        <x:v>BRONZE</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>INSUFFICIENT_ACTUAL_HISTORY</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>Avoid unstable short samples</x:v>
+        <x:v>Primary</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>Model disabled until enough actual history</x:v>
+        <x:v>Best available data</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Holdout window</x:v>
-      </x:c>
-      <x:c r="B5" s="18" t="n">
-        <x:v>20</x:v>
+        <x:v>Model build</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Bronze coverage &lt;60%</x:v>
       </x:c>
       <x:c r="C5" t="str">
+        <x:v>Replace ticker with config fallback</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>BaseVulnerability</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
         <x:v>ASSUMPTION</x:v>
       </x:c>
-      <x:c r="D5" t="str">
-        <x:v>Forecast selection</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>Last 20 days</x:v>
-      </x:c>
       <x:c r="F5" t="str">
-        <x:v>N/A</x:v>
+        <x:v>FALLBACK</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>Backtest</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>Real out-of-sample check</x:v>
+        <x:v>Ticker-level</x:v>
       </x:c>
       <x:c r="I5" t="str">
-        <x:v>Closer to production use</x:v>
+        <x:v>Explicit assumption</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>ARIMA vs Naive</x:v>
-      </x:c>
-      <x:c r="B6" s="18" t="str">
-        <x:v>RMSE</x:v>
+        <x:v>Model build</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Unexpected null after merge</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>MODEL</x:v>
+        <x:v>Rehydrate ticker from config</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>LPI/Interbank</x:v>
+        <x:v>BaseVulnerability</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>ARIMA RMSE &lt; Naive RMSE</x:v>
+        <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Use Naive</x:v>
+        <x:v>FALLBACK</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>OK_BENCHMARK</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>Never publish a worse complex model</x:v>
+        <x:v>Absolute guarantee</x:v>
       </x:c>
       <x:c r="I6" t="str">
-        <x:v>Flat forecast can be the correct production choice</x:v>
+        <x:v>Prevents blank model output</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Confidence HIGH</x:v>
-      </x:c>
-      <x:c r="B7" s="18" t="str">
-        <x:v>Skill &gt;=20%</x:v>
+        <x:v>Streamlit runtime</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>bank_stress_forecast missing/null</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>MODEL</x:v>
+        <x:v>Build fallback in app from config</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Stress + Stress Lab</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Pass</x:v>
+        <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>N/A</x:v>
+        <x:v>FALLBACK</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>HIGH</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>Strong incremental value</x:v>
+        <x:v>Second safety net</x:v>
       </x:c>
       <x:c r="I7" t="str">
-        <x:v>Higher confidence</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Confidence MEDIUM</x:v>
-      </x:c>
-      <x:c r="B8" s="18" t="str">
-        <x:v>Skill 5–20%</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>MODEL</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>Forecast</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>Pass</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>MEDIUM</x:v>
-      </x:c>
-      <x:c r="H8" t="str">
-        <x:v>Moderate incremental value</x:v>
-      </x:c>
-      <x:c r="I8" t="str">
-        <x:v>Use with caution</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>Confidence LOW</x:v>
-      </x:c>
-      <x:c r="B9" s="18" t="str">
-        <x:v>Skill &lt;5% or benchmark</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>MODEL</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>Forecast</x:v>
-      </x:c>
-      <x:c r="E9" t="str">
-        <x:v>Fail/weak</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>Use benchmark</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>LOW</x:v>
-      </x:c>
-      <x:c r="H9" t="str">
-        <x:v>Little incremental value</x:v>
-      </x:c>
-      <x:c r="I9" t="str">
-        <x:v>Do not over-interpret point estimate</x:v>
+        <x:v>Dashboard remains usable</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -663,20 +598,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="44" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="50" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>BANK FUNDING STRESS — DATA GATE &amp; TRANSMISSION</x:v>
+        <x:v>FORECAST SELECTION &amp; CONFIDENCE</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -689,224 +624,205 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>Factor</x:v>
+        <x:v>Rule</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
-        <x:v>Source priority</x:v>
+        <x:v>Threshold/Method</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
-        <x:v>Rule</x:v>
+        <x:v>Target</x:v>
       </x:c>
       <x:c r="D3" s="10" t="str">
-        <x:v>Stress direction</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
-        <x:v>Coverage role</x:v>
+        <x:v>Fail</x:v>
       </x:c>
       <x:c r="F3" s="10" t="str">
-        <x:v>Data Type</x:v>
+        <x:v>Production model</x:v>
       </x:c>
       <x:c r="G3" s="10" t="str">
-        <x:v>Fallback</x:v>
+        <x:v>Confidence</x:v>
       </x:c>
       <x:c r="H3" s="10" t="str">
-        <x:v>Output</x:v>
+        <x:v>Why</x:v>
       </x:c>
       <x:c r="I3" s="10" t="str">
-        <x:v>Notes</x:v>
+        <x:v>User message</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>LDR</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>Bronze → fallback</x:v>
+        <x:v>Minimum history</x:v>
+      </x:c>
+      <x:c r="B4" s="18" t="n">
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>35 × (LDR−85%)</x:v>
+        <x:v>LPI / Interbank</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>Higher = more stress</x:v>
+        <x:v>Continue</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>1/5</x:v>
+        <x:v>No forecast</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>ACTUAL/ASSUMPTION</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>Ticker-level</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>BaseVulnerability</x:v>
-      </x:c>
-      <x:c r="I4" t="str"/>
+        <x:v>Avoid unstable small sample</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Insufficient actual history</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>CASA</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Bronze → fallback</x:v>
+        <x:v>Holdout</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="str">
+        <x:v>20 days</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>−25 × (CASA−20%)</x:v>
+        <x:v>Candidate selection</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Higher = less stress</x:v>
+        <x:v>Evaluate ARIMA</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>1/5</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>ACTUAL/ASSUMPTION</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>Ticker-level</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>BaseVulnerability</x:v>
-      </x:c>
-      <x:c r="I5" t="str"/>
+        <x:v>Out-of-sample test</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Backtest</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>InterbankDep</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>Bronze → fallback</x:v>
+        <x:v>ARIMA vs Naive</x:v>
+      </x:c>
+      <x:c r="B6" s="18" t="str">
+        <x:v>RMSE</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>45 × ratio</x:v>
+        <x:v>LPI / Interbank</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Higher = more stress</x:v>
+        <x:v>ARIMA RMSE &lt; Naive</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>1/5</x:v>
+        <x:v>ARIMA RMSE &gt;= Naive</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>ACTUAL/ASSUMPTION</x:v>
+        <x:v>NAIVE_RANDOM_WALK</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>Ticker-level</x:v>
+        <x:v>LOW on fail</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>BaseVulnerability</x:v>
-      </x:c>
-      <x:c r="I6" t="str"/>
+        <x:v>Never publish worse complexity</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Benchmark selected if ARIMA underperforms</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>CreditDepositGap</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Bronze → fallback</x:v>
+        <x:v>Skill &gt;=20%</x:v>
+      </x:c>
+      <x:c r="B7" s="18" t="str">
+        <x:v>1-RMSE/NaiveRMSE</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>30 × gap</x:v>
+        <x:v>Forecast</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Higher = more stress</x:v>
+        <x:v>HIGH</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>1/5</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>ACTUAL/ASSUMPTION</x:v>
+        <x:v>ARIMA</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>Ticker-level</x:v>
+        <x:v>HIGH</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>BaseVulnerability</x:v>
-      </x:c>
-      <x:c r="I7" t="str"/>
+        <x:v>Strong incremental value</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Higher confidence</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>NIM</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Bronze → fallback</x:v>
+        <x:v>Skill 5–20%</x:v>
+      </x:c>
+      <x:c r="B8" s="18" t="str">
+        <x:v>1-RMSE/NaiveRMSE</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>−10 × (NIM−3%)</x:v>
+        <x:v>Forecast</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>Higher = less stress</x:v>
+        <x:v>MEDIUM</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>1/5</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>ACTUAL/ASSUMPTION</x:v>
+        <x:v>ARIMA</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>Ticker-level</x:v>
+        <x:v>MEDIUM</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>BaseVulnerability</x:v>
-      </x:c>
-      <x:c r="I8" t="str"/>
+        <x:v>Moderate value</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Use with caution</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Bronze gate</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>MetricCoverage</x:v>
+        <x:v>Skill &lt;5%</x:v>
+      </x:c>
+      <x:c r="B9" s="18" t="str">
+        <x:v>1-RMSE/NaiveRMSE</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>&gt;=60% (3/5)</x:v>
+        <x:v>Forecast</x:v>
       </x:c>
       <x:c r="D9" t="str">
+        <x:v>LOW</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
         <x:v>N/A</x:v>
       </x:c>
-      <x:c r="E9" t="str">
-        <x:v>Gate</x:v>
-      </x:c>
       <x:c r="F9" t="str">
-        <x:v>MODEL</x:v>
+        <x:v>ARIMA/Benchmark</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>Fallback whole ticker if fail</x:v>
+        <x:v>LOW</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>Use ACTUAL only if pass</x:v>
+        <x:v>Little incremental value</x:v>
       </x:c>
       <x:c r="I9" t="str">
-        <x:v>Prevents blank/false-precision bars</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>System LPI</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Forecast</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>Multiplier = 1+0.15×max(LPI,0)</x:v>
-      </x:c>
-      <x:c r="D10" t="str">
-        <x:v>Higher = more stress</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>MODEL</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="H10" t="str">
-        <x:v>StressVulnerability</x:v>
-      </x:c>
-      <x:c r="I10" t="str">
-        <x:v>Scenario transmission</x:v>
+        <x:v>Do not over-interpret point estimate</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -927,14 +843,11 @@
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="60" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>TRUE INTERBANK ACTUAL INPUT — OPTIONAL FALLBACK</x:v>
+        <x:v>TRUE INTERBANK ACTUAL INPUT — OPTIONAL</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -961,19 +874,10 @@
       <x:c r="F3" s="10" t="str">
         <x:v>Instruction</x:v>
       </x:c>
-      <x:c r="H3" s="10" t="str">
-        <x:v>Export rule</x:v>
-      </x:c>
-      <x:c r="I3" s="10" t="str">
-        <x:v>Value</x:v>
-      </x:c>
-      <x:c r="J3" s="10" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="22"/>
-      <x:c r="B4" s="20"/>
+      <x:c r="A4" s="20"/>
+      <x:c r="B4" s="22"/>
       <x:c r="C4" s="18"/>
       <x:c r="D4" s="18"/>
       <x:c r="E4" s="18" t="str">
@@ -982,19 +886,10 @@
       <x:c r="F4" t="str">
         <x:v>Enter only published ACTUAL observations; keep source URL.</x:v>
       </x:c>
-      <x:c r="H4" t="str">
-        <x:v>Minimum valid rows</x:v>
-      </x:c>
-      <x:c r="I4" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="J4" t="str">
-        <x:v>Below this, existing interbank_manual.csv is NOT overwritten</x:v>
-      </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="22"/>
-      <x:c r="B5" s="20"/>
+      <x:c r="A5" s="20"/>
+      <x:c r="B5" s="22"/>
       <x:c r="C5" s="18"/>
       <x:c r="D5" s="18"/>
       <x:c r="E5" s="18" t="str">
@@ -1003,19 +898,10 @@
       <x:c r="F5" t="str">
         <x:v>Enter only published ACTUAL observations; keep source URL.</x:v>
       </x:c>
-      <x:c r="H5" t="str">
-        <x:v>Data Type</x:v>
-      </x:c>
-      <x:c r="I5" t="str">
-        <x:v>ACTUAL</x:v>
-      </x:c>
-      <x:c r="J5" t="str">
-        <x:v>Assumptions are rejected</x:v>
-      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="22"/>
-      <x:c r="B6" s="20"/>
+      <x:c r="A6" s="20"/>
+      <x:c r="B6" s="22"/>
       <x:c r="C6" s="18"/>
       <x:c r="D6" s="18"/>
       <x:c r="E6" s="18" t="str">
@@ -1024,19 +910,10 @@
       <x:c r="F6" t="str">
         <x:v>Enter only published ACTUAL observations; keep source URL.</x:v>
       </x:c>
-      <x:c r="H6" t="str">
-        <x:v>Source URL</x:v>
-      </x:c>
-      <x:c r="I6" t="str">
-        <x:v>Required</x:v>
-      </x:c>
-      <x:c r="J6" t="str">
-        <x:v>Must start with http</x:v>
-      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="22"/>
-      <x:c r="B7" s="20"/>
+      <x:c r="A7" s="20"/>
+      <x:c r="B7" s="22"/>
       <x:c r="C7" s="18"/>
       <x:c r="D7" s="18"/>
       <x:c r="E7" s="18" t="str">
@@ -1045,19 +922,10 @@
       <x:c r="F7" t="str">
         <x:v>Enter only published ACTUAL observations; keep source URL.</x:v>
       </x:c>
-      <x:c r="H7" t="str">
-        <x:v>Priority 1</x:v>
-      </x:c>
-      <x:c r="I7" t="str">
-        <x:v>Bronze true interbank</x:v>
-      </x:c>
-      <x:c r="J7" t="str">
-        <x:v>Used before manual/public input</x:v>
-      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="22"/>
-      <x:c r="B8" s="20"/>
+      <x:c r="A8" s="20"/>
+      <x:c r="B8" s="22"/>
       <x:c r="C8" s="18"/>
       <x:c r="D8" s="18"/>
       <x:c r="E8" s="18" t="str">
@@ -1066,19 +934,10 @@
       <x:c r="F8" t="str">
         <x:v>Enter only published ACTUAL observations; keep source URL.</x:v>
       </x:c>
-      <x:c r="H8" t="str">
-        <x:v>Proxy</x:v>
-      </x:c>
-      <x:c r="I8" t="str">
-        <x:v>Not allowed</x:v>
-      </x:c>
-      <x:c r="J8" t="str">
-        <x:v>Deposit/lending rates are never relabelled as interbank</x:v>
-      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="22"/>
-      <x:c r="B9" s="20"/>
+      <x:c r="A9" s="20"/>
+      <x:c r="B9" s="22"/>
       <x:c r="C9" s="18"/>
       <x:c r="D9" s="18"/>
       <x:c r="E9" s="18" t="str">
@@ -1089,8 +948,8 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="22"/>
-      <x:c r="B10" s="20"/>
+      <x:c r="A10" s="20"/>
+      <x:c r="B10" s="22"/>
       <x:c r="C10" s="18"/>
       <x:c r="D10" s="18"/>
       <x:c r="E10" s="18" t="str">
@@ -1101,8 +960,8 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="22"/>
-      <x:c r="B11" s="20"/>
+      <x:c r="A11" s="20"/>
+      <x:c r="B11" s="22"/>
       <x:c r="C11" s="18"/>
       <x:c r="D11" s="18"/>
       <x:c r="E11" s="18" t="str">
@@ -1113,8 +972,8 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="22"/>
-      <x:c r="B12" s="20"/>
+      <x:c r="A12" s="20"/>
+      <x:c r="B12" s="22"/>
       <x:c r="C12" s="18"/>
       <x:c r="D12" s="18"/>
       <x:c r="E12" s="18" t="str">
@@ -1125,8 +984,8 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="22"/>
-      <x:c r="B13" s="20"/>
+      <x:c r="A13" s="20"/>
+      <x:c r="B13" s="22"/>
       <x:c r="C13" s="18"/>
       <x:c r="D13" s="18"/>
       <x:c r="E13" s="18" t="str">
@@ -1137,8 +996,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="22"/>
-      <x:c r="B14" s="20"/>
+      <x:c r="A14" s="20"/>
+      <x:c r="B14" s="22"/>
       <x:c r="C14" s="18"/>
       <x:c r="D14" s="18"/>
       <x:c r="E14" s="18" t="str">
@@ -1149,8 +1008,8 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="22"/>
-      <x:c r="B15" s="20"/>
+      <x:c r="A15" s="20"/>
+      <x:c r="B15" s="22"/>
       <x:c r="C15" s="18"/>
       <x:c r="D15" s="18"/>
       <x:c r="E15" s="18" t="str">
@@ -1161,8 +1020,8 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="22"/>
-      <x:c r="B16" s="20"/>
+      <x:c r="A16" s="20"/>
+      <x:c r="B16" s="22"/>
       <x:c r="C16" s="18"/>
       <x:c r="D16" s="18"/>
       <x:c r="E16" s="18" t="str">
@@ -1173,8 +1032,8 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="22"/>
-      <x:c r="B17" s="20"/>
+      <x:c r="A17" s="20"/>
+      <x:c r="B17" s="22"/>
       <x:c r="C17" s="18"/>
       <x:c r="D17" s="18"/>
       <x:c r="E17" s="18" t="str">
@@ -1185,8 +1044,8 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="22"/>
-      <x:c r="B18" s="20"/>
+      <x:c r="A18" s="20"/>
+      <x:c r="B18" s="22"/>
       <x:c r="C18" s="18"/>
       <x:c r="D18" s="18"/>
       <x:c r="E18" s="18" t="str">
@@ -1197,8 +1056,8 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="22"/>
-      <x:c r="B19" s="20"/>
+      <x:c r="A19" s="20"/>
+      <x:c r="B19" s="22"/>
       <x:c r="C19" s="18"/>
       <x:c r="D19" s="18"/>
       <x:c r="E19" s="18" t="str">
@@ -1209,8 +1068,8 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="22"/>
-      <x:c r="B20" s="20"/>
+      <x:c r="A20" s="20"/>
+      <x:c r="B20" s="22"/>
       <x:c r="C20" s="18"/>
       <x:c r="D20" s="18"/>
       <x:c r="E20" s="18" t="str">
@@ -1221,8 +1080,8 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="22"/>
-      <x:c r="B21" s="20"/>
+      <x:c r="A21" s="20"/>
+      <x:c r="B21" s="22"/>
       <x:c r="C21" s="18"/>
       <x:c r="D21" s="18"/>
       <x:c r="E21" s="18" t="str">
@@ -1233,8 +1092,8 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="22"/>
-      <x:c r="B22" s="20"/>
+      <x:c r="A22" s="20"/>
+      <x:c r="B22" s="22"/>
       <x:c r="C22" s="18"/>
       <x:c r="D22" s="18"/>
       <x:c r="E22" s="18" t="str">
@@ -1245,8 +1104,8 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="22"/>
-      <x:c r="B23" s="20"/>
+      <x:c r="A23" s="20"/>
+      <x:c r="B23" s="22"/>
       <x:c r="C23" s="18"/>
       <x:c r="D23" s="18"/>
       <x:c r="E23" s="18" t="str">
@@ -1257,8 +1116,8 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="22"/>
-      <x:c r="B24" s="20"/>
+      <x:c r="A24" s="20"/>
+      <x:c r="B24" s="22"/>
       <x:c r="C24" s="18"/>
       <x:c r="D24" s="18"/>
       <x:c r="E24" s="18" t="str">
@@ -1269,8 +1128,8 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="22"/>
-      <x:c r="B25" s="20"/>
+      <x:c r="A25" s="20"/>
+      <x:c r="B25" s="22"/>
       <x:c r="C25" s="18"/>
       <x:c r="D25" s="18"/>
       <x:c r="E25" s="18" t="str">
@@ -1281,8 +1140,8 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="22"/>
-      <x:c r="B26" s="20"/>
+      <x:c r="A26" s="20"/>
+      <x:c r="B26" s="22"/>
       <x:c r="C26" s="18"/>
       <x:c r="D26" s="18"/>
       <x:c r="E26" s="18" t="str">
@@ -1293,8 +1152,8 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="22"/>
-      <x:c r="B27" s="20"/>
+      <x:c r="A27" s="20"/>
+      <x:c r="B27" s="22"/>
       <x:c r="C27" s="18"/>
       <x:c r="D27" s="18"/>
       <x:c r="E27" s="18" t="str">
@@ -1305,8 +1164,8 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="22"/>
-      <x:c r="B28" s="20"/>
+      <x:c r="A28" s="20"/>
+      <x:c r="B28" s="22"/>
       <x:c r="C28" s="18"/>
       <x:c r="D28" s="18"/>
       <x:c r="E28" s="18" t="str">
@@ -1317,8 +1176,8 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="22"/>
-      <x:c r="B29" s="20"/>
+      <x:c r="A29" s="20"/>
+      <x:c r="B29" s="22"/>
       <x:c r="C29" s="18"/>
       <x:c r="D29" s="18"/>
       <x:c r="E29" s="18" t="str">
@@ -1329,8 +1188,8 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="22"/>
-      <x:c r="B30" s="20"/>
+      <x:c r="A30" s="20"/>
+      <x:c r="B30" s="22"/>
       <x:c r="C30" s="18"/>
       <x:c r="D30" s="18"/>
       <x:c r="E30" s="18" t="str">
@@ -1341,8 +1200,8 @@
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="22"/>
-      <x:c r="B31" s="20"/>
+      <x:c r="A31" s="20"/>
+      <x:c r="B31" s="22"/>
       <x:c r="C31" s="18"/>
       <x:c r="D31" s="18"/>
       <x:c r="E31" s="18" t="str">
@@ -1353,8 +1212,8 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="22"/>
-      <x:c r="B32" s="20"/>
+      <x:c r="A32" s="20"/>
+      <x:c r="B32" s="22"/>
       <x:c r="C32" s="18"/>
       <x:c r="D32" s="18"/>
       <x:c r="E32" s="18" t="str">
@@ -1365,8 +1224,8 @@
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="22"/>
-      <x:c r="B33" s="20"/>
+      <x:c r="A33" s="20"/>
+      <x:c r="B33" s="22"/>
       <x:c r="C33" s="18"/>
       <x:c r="D33" s="18"/>
       <x:c r="E33" s="18" t="str">
@@ -1388,18 +1247,19 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>SAFE CODE-ONLY UPGRADE CHECKLIST</x:v>
+        <x:v>PRODUCTION R3 VALIDATION TEST</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -1407,171 +1267,137 @@
       <x:c r="E1" s="14"/>
       <x:c r="F1" s="14"/>
       <x:c r="G1" s="14"/>
+      <x:c r="H1" s="14"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>Step</x:v>
+        <x:v>Test</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
-        <x:v>Action</x:v>
+        <x:v>Input state</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
-        <x:v>data/</x:v>
+        <x:v>Expected</x:v>
       </x:c>
       <x:c r="D3" s="10" t="str">
-        <x:v>Command / file</x:v>
+        <x:v>Observed</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
-        <x:v>Expected result</x:v>
+        <x:v>Status</x:v>
       </x:c>
       <x:c r="F3" s="10" t="str">
-        <x:v>Risk if skipped</x:v>
+        <x:v>Implication</x:v>
       </x:c>
       <x:c r="G3" s="10" t="str">
-        <x:v>Status</x:v>
+        <x:v>Data Type</x:v>
+      </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="n">
-        <x:v>1</x:v>
+      <x:c r="A4" t="str">
+        <x:v>Stress fallback</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>KEEP existing production data folder</x:v>
+        <x:v>20 Bronze bank rows; all 5 stress metrics null</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>KEEP</x:v>
+        <x:v>20 valid BaseVulnerability rows</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>data/</x:v>
+        <x:v>20 valid rows</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>Bronze ACTUAL + model history preserved</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>NO_LPI / loss of actual history</x:v>
+        <x:v>Stress charts cannot be blank</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>REQUIRED</x:v>
+        <x:v>ASSUMPTION fallback</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Automated package test</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="n">
-        <x:v>2</x:v>
+      <x:c r="A5" t="str">
+        <x:v>Fallback source</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Copy code-only package files</x:v>
+        <x:v>Bronze coverage = 0</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>KEEP</x:v>
+        <x:v>All 20 tickers use fallback</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>app.py, scripts/, config/, *.bat, Master</x:v>
+        <x:v>20 FALLBACK</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>Code upgraded</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>None</x:v>
+        <x:v>Transparent lineage</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>REQUIRED</x:v>
-      </x:c>
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="H5" t="str"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="n">
-        <x:v>3</x:v>
+      <x:c r="A6" t="str">
+        <x:v>Interbank absence</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Git code upgrade</x:v>
+        <x:v>No true interbank</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>KEEP</x:v>
+        <x:v>No ON forecast</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>git add -A / commit / push</x:v>
+        <x:v>NO_INTERBANK_DATA</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>Streamlit code redeploys</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Old code remains</x:v>
+        <x:v>No fabricated rate</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>REQUIRED</x:v>
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Funding proxy may display separately</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="n">
-        <x:v>4</x:v>
+      <x:c r="A7" t="str">
+        <x:v>Package safety</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Run Bronze refresh/model build</x:v>
+        <x:v>Upgrade artifact</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>KEEP</x:v>
+        <x:v>No data/ files</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>REFRESH_BRONZE_BUILD_MODELS_AND_PUSH.bat</x:v>
+        <x:v>0 data/ files</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>New outputs generated and pushed</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Stale diagnostics/stress</x:v>
+        <x:v>Preserves production Bronze data</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>REQUIRED</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Review Diagnostics</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>KEEP</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>Streamlit Diagnostics tab</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>Check coverage/model governance</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>False confidence</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>If interbank missing</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>KEEP</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>INTERBANK_INPUT sheet</x:v>
-      </x:c>
-      <x:c r="E9" t="str">
-        <x:v>Provide actual public series if available</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>No ON forecast</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>OPTIONAL</x:v>
-      </x:c>
+        <x:v>CONTROL</x:v>
+      </x:c>
+      <x:c r="H7" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1581,15 +1407,185 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="50" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="14" t="str">
+        <x:v>SAFE CODE-ONLY UPGRADE</x:v>
+      </x:c>
+      <x:c r="B1" s="14"/>
+      <x:c r="C1" s="14"/>
+      <x:c r="D1" s="14"/>
+      <x:c r="E1" s="14"/>
+      <x:c r="F1" s="14"/>
+      <x:c r="G1" s="14"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="10" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>Keep data/?</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>Files / command</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>Expected result</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>Risk if skipped</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Keep existing repository data folder</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>data/</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Bronze ACTUAL and history preserved</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Loss of production data</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Copy code-only R3 package</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>app.py, scripts/, config/, *.bat, Master</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>R3 code active</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Old bugs remain</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Push code</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>git add -A / commit / push</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Streamlit redeploys</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Cloud still old code</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Run local refresh/model BAT</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>REFRESH_BRONZE_BUILD_MODELS_AND_PUSH.bat</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>New model outputs pushed</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Stale bank stress output</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Review Stress diagnostics</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Diagnostics tab</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>20 valid BaseVulnerability minimum</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Potential stale output</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>REVIEW</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>PRODUCTION R2 CONTROL PANEL</x:v>
+        <x:v>PRODUCTION R3 CONTROL PANEL</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1645,85 +1641,99 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Bank actual coverage gate</x:v>
-      </x:c>
-      <x:c r="B6" s="24" t="n">
-        <x:v>0.6</x:v>
+        <x:v>Stress safety layers</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>ASSUMPTION</x:v>
+        <x:v>CONTROL</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>At least 3/5 core metrics</x:v>
+        <x:v>Model + runtime fallback</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>LPI minimum drivers</x:v>
+        <x:v>Fallback universe</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>At least two ACTUAL components</x:v>
+        <x:v>20 banks if Bronze stress metrics unavailable</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Daily forecast minimum obs</x:v>
-      </x:c>
-      <x:c r="B8" s="18" t="n">
-        <x:v>80</x:v>
+        <x:v>Bank actual coverage gate</x:v>
+      </x:c>
+      <x:c r="B8" s="24" t="n">
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>Production gate</x:v>
+        <x:v>At least 3/5 core metrics</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Holdout days</x:v>
+        <x:v>LPI minimum drivers</x:v>
       </x:c>
       <x:c r="B9" s="18" t="n">
-        <x:v>20</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>Model selection</x:v>
+        <x:v>At least two ACTUAL components</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>ARIMA can underperform naive?</x:v>
+        <x:v>Daily forecast minimum obs</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>CONTROL</x:v>
+        <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>If yes, benchmark is selected instead</x:v>
+        <x:v>Production forecast gate</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Manual interbank min rows</x:v>
+        <x:v>Holdout days</x:v>
       </x:c>
       <x:c r="B11" s="18" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" t="str">
         <x:v>ASSUMPTION</x:v>
       </x:c>
       <x:c r="D11" t="str">
+        <x:v>Model selection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Manual interbank min rows</x:v>
+      </x:c>
+      <x:c r="B12" s="18" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
         <x:v>Protect existing actual file</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Upgrade liquidity intelligence R7 data pipeline hardening
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb28a979b3658470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6_SCHEMA_MAP" sheetId="2" r:id="R26b0d01fb44c402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_LOGIC" sheetId="3" r:id="Rbb284c733f7b4581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPGRADE_CHECKLIST" sheetId="4" r:id="R00fb4489fb2d4b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfabd298efef54ce7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6_SCHEMA_MAP" sheetId="2" r:id="R852e549ef5a74b8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_LOGIC" sheetId="3" r:id="Rf16368cc527b4f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPGRADE_CHECKLIST" sheetId="4" r:id="R87a0574821274233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R7_HARDENING" sheetId="5" r:id="Rad24b7f881d748af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34,12 +35,22 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2747"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -59,7 +70,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -88,6 +99,21 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1015,4 +1041,462 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="46" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="44" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="23" t="str">
+        <x:v>R7 — DATA PIPELINE HARDENING</x:v>
+      </x:c>
+      <x:c r="B1" s="23"/>
+      <x:c r="C1" s="23"/>
+      <x:c r="D1" s="23"/>
+      <x:c r="E1" s="23"/>
+      <x:c r="F1" s="23"/>
+      <x:c r="G1" s="23"/>
+      <x:c r="H1" s="23"/>
+      <x:c r="I1" s="23"/>
+      <x:c r="J1" s="23"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="22" t="str">
+        <x:v>Issue</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str">
+        <x:v>R6 symptom</x:v>
+      </x:c>
+      <x:c r="C3" s="22" t="str">
+        <x:v>R7 root fix</x:v>
+      </x:c>
+      <x:c r="D3" s="22" t="str">
+        <x:v>Primary data source</x:v>
+      </x:c>
+      <x:c r="E3" s="22" t="str">
+        <x:v>Fallback policy</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="str">
+        <x:v>Production label</x:v>
+      </x:c>
+      <x:c r="G3" s="22" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="H3" s="22" t="str">
+        <x:v>Expected effect</x:v>
+      </x:c>
+      <x:c r="I3" s="22" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+      <x:c r="J3" s="22" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Interbank backend</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>interest_rate length=3650 → HTTP 500</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Progressive request 365→180→90; stop on first true ON series</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Vnstock interest_rate() filtered Interbank/Qua đêm</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Manual ACTUAL or prior ACTUAL only</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>BRONZE / MANUAL_ACTUAL</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Observation count + latest date</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Interbank ACTUAL should load without oversized request</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>No deposit/lending substitution</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Official docs example length=365</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Bank coverage</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>0 banks &gt;=60% caused full ticker fallback</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Field-level fallback: preserve every actual metric and fill only missing fields</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Fundamental tidy data / Semantic ID</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Per-field assumption only</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>BRONZE / HYBRID / FALLBACK</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>ActualMetricCount + MetricCoverage</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Actual LDR/CASA etc. are no longer discarded</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Lineage visible per ticker</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>HYBRID = 1–4/5 actual metrics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Statsmodels warnings</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>unsupported index repeated</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Convert training series to RangeIndex before SARIMAX</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Model input</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>No index warnings expected</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Cleaner logs; same forecast-date output</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Forecast dates added after model</x:v>
+      </x:c>
+      <x:c r="J6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Budget 404</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Non-core error noise</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Mark budget as DEGRADED and do not block pipeline</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Vnstock macro</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>DEGRADED</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Status log only</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Core model unaffected</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Non-core dataset</x:v>
+      </x:c>
+      <x:c r="J7" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="24" t="str">
+        <x:v>R7 STRESS DATA LINEAGE</x:v>
+      </x:c>
+      <x:c r="B9" s="24"/>
+      <x:c r="C9" s="24"/>
+      <x:c r="D9" s="24"/>
+      <x:c r="E9" s="24"/>
+      <x:c r="F9" s="24"/>
+      <x:c r="G9" s="24"/>
+      <x:c r="H9" s="24"/>
+      <x:c r="I9" s="24"/>
+      <x:c r="J9" s="24"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="22" t="str">
+        <x:v>Source Mode</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>Actual metric count</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>Assumption metric count</x:v>
+      </x:c>
+      <x:c r="D10" s="22" t="str">
+        <x:v>Data Type</x:v>
+      </x:c>
+      <x:c r="E10" s="22" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="str">
+        <x:v>Can score?</x:v>
+      </x:c>
+      <x:c r="G10" s="22" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="H10" s="22" t="str">
+        <x:v>Color convention</x:v>
+      </x:c>
+      <x:c r="I10" s="22" t="str">
+        <x:v>User interpretation</x:v>
+      </x:c>
+      <x:c r="J10" s="22" t="str">
+        <x:v>Example</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>BRONZE</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>All five stress metrics are actual</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Green lineage</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Highest-quality bank stress row</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>All LDR/CASA/IB/Gap/NIM actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>HYBRID</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>1–4</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>4–1</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Keep actual fields; fill only missing fields</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Mixed lineage</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Partly actual, partly assumption</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Actual LDR/CASA + assumed NIM/gap</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>FALLBACK</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>No actual stress fields available</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Assumption lineage</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>Scenario only; not an empirical bank conclusion</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>All five from config</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="24" t="str">
+        <x:v>INTERBANK REQUEST LADDER</x:v>
+      </x:c>
+      <x:c r="B15" s="24"/>
+      <x:c r="C15" s="24"/>
+      <x:c r="D15" s="24"/>
+      <x:c r="E15" s="24"/>
+      <x:c r="F15" s="24"/>
+      <x:c r="G15" s="24"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>Call</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>Why</x:v>
+      </x:c>
+      <x:c r="D16" s="22" t="str">
+        <x:v>Stop condition</x:v>
+      </x:c>
+      <x:c r="E16" s="22" t="str">
+        <x:v>Expected observations</x:v>
+      </x:c>
+      <x:c r="F16" s="22" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="G16" s="22" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>interest_rate(period='day', length=365)</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Official-sized request; avoids 3650-day backend overload</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>ON rows found</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>&gt;=80 preferred</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Use first successful true interbank series</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>interest_rate(length=365)</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Runtime compatibility</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>ON rows found</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>&gt;=80 preferred</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="G18" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>180-day variants</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Reduce backend payload</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>ON rows found</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>&gt;=80 preferred</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="G19" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>90-day variants</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Last Bronze attempt</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>ON rows found</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>&gt;=80 ideal; otherwise chart only</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="G20" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A9:J9"/>
+    <x:mergeCell ref="A15:G15"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Upgrade liquidity intelligence R8 MultiIndex safe
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfabd298efef54ce7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6_SCHEMA_MAP" sheetId="2" r:id="R852e549ef5a74b8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_LOGIC" sheetId="3" r:id="Rf16368cc527b4f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPGRADE_CHECKLIST" sheetId="4" r:id="R87a0574821274233"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R7_HARDENING" sheetId="5" r:id="Rad24b7f881d748af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R144f78d688ee417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6_SCHEMA_MAP" sheetId="2" r:id="Rceaa76a80aec4586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_LOGIC" sheetId="3" r:id="R5a0b62b6309e4bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPGRADE_CHECKLIST" sheetId="4" r:id="R8b509e6a5fa94bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R7_HARDENING" sheetId="5" r:id="R4868774849364593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R8_MULTIINDEX_FIX" sheetId="6" r:id="R454764b58a924def"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35,12 +36,22 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2747"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -70,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -114,6 +125,21 @@
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1499,4 +1525,313 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="32" t="str">
+        <x:v>R8 — MULTIINDEX-SAFE DATA FIX</x:v>
+      </x:c>
+      <x:c r="B1" s="32"/>
+      <x:c r="C1" s="32"/>
+      <x:c r="D1" s="32"/>
+      <x:c r="E1" s="32"/>
+      <x:c r="F1" s="32"/>
+      <x:c r="G1" s="32"/>
+      <x:c r="H1" s="32"/>
+      <x:c r="I1" s="32"/>
+      <x:c r="J1" s="32"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="31" t="str">
+        <x:v>Issue</x:v>
+      </x:c>
+      <x:c r="B3" s="31" t="str">
+        <x:v>Observed R7 log</x:v>
+      </x:c>
+      <x:c r="C3" s="31" t="str">
+        <x:v>Root cause</x:v>
+      </x:c>
+      <x:c r="D3" s="31" t="str">
+        <x:v>R8 fix</x:v>
+      </x:c>
+      <x:c r="E3" s="31" t="str">
+        <x:v>Primary source</x:v>
+      </x:c>
+      <x:c r="F3" s="31" t="str">
+        <x:v>Fallback</x:v>
+      </x:c>
+      <x:c r="G3" s="31" t="str">
+        <x:v>Expected status</x:v>
+      </x:c>
+      <x:c r="H3" s="31" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="I3" s="31" t="str">
+        <x:v>Production impact</x:v>
+      </x:c>
+      <x:c r="J3" s="31" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Bank Fundamental</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>20/20 banks ERROR: isna is not defined for MultiIndex</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>One Fundamental source failure aborted whole ticker; runtime dataframe/index can be MultiIndex</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Isolate health/ratio/BS calls; MultiIndex-safe flattening; financial_health primary; remove drop_empty=False</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Vnstock Fundamental</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Field-level HYBRID/FALLBACK</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Bank rows should be OK/PARTIAL, not ERROR</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>ActualMetricCount + ParserCall</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Bronze metrics can survive partial source failures</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>financial_health scorecard='bank'</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Interbank</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>365 rows returned but no ON match</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Parser assumed simple columns; Vietnamese 'đ' normalization also failed</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Flatten MultiIndex + scan all text columns + explicit đ→d normalization + dynamic date/value detection</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Vnstock interest_rate()</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Prior/manual ACTUAL only</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>OK_INTEREST_RATE_FILTER if ON exists</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Observation count + latest date</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Interbank ACTUAL should populate</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>365→180→90 request ladder retained</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Statsmodels</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>unsupported index warning remained</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>MarkovRegression still received gapped index</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>RangeIndex also applied to Markov regime</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Model input</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>No unsupported-index warning</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Log scan</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Cleaner model build</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Forecast governance unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="33" t="str">
+        <x:v>R8 DATA SOURCE ISOLATION</x:v>
+      </x:c>
+      <x:c r="B8" s="33"/>
+      <x:c r="C8" s="33"/>
+      <x:c r="D8" s="33"/>
+      <x:c r="E8" s="33"/>
+      <x:c r="F8" s="33"/>
+      <x:c r="G8" s="33"/>
+      <x:c r="H8" s="33"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="31" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B9" s="31" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="C9" s="31" t="str">
+        <x:v>If success</x:v>
+      </x:c>
+      <x:c r="D9" s="31" t="str">
+        <x:v>If failure</x:v>
+      </x:c>
+      <x:c r="E9" s="31" t="str">
+        <x:v>Metrics expected</x:v>
+      </x:c>
+      <x:c r="F9" s="31" t="str">
+        <x:v>Can ticker continue?</x:v>
+      </x:c>
+      <x:c r="G9" s="31" t="str">
+        <x:v>Output lineage</x:v>
+      </x:c>
+      <x:c r="H9" s="31" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>financial_health(scorecard='bank')</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Parse LDR/CASA/NIM first</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Record source error only</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>LDR, CASA, NIM</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>ACTUAL fields retained</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Stable scorecard source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>ratio()</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Fill missing LDR/CASA/NIM</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Continue with health/BS</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>LDR, CASA, NIM</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>ACTUAL fields retained</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Source isolated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>balance_sheet()</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Compute loans/deposits/interbank ratios</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Continue without BS metrics</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Loans, deposits, assets, interbank liabilities</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>HYBRID if needed</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Source isolated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>config fallback</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Fill only missing fields</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>Any missing stress metric</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>HYBRID/FALLBACK</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Never overwrites an actual field</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A8:H8"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Upgrade CASA actual sources and interbank history
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,11 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc242bd2d3104499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_CONFIG" sheetId="2" r:id="R01cb99d84abd48ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ASSUMPTIONS" sheetId="3" r:id="R1385f8d2edce4336"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_INPUT" sheetId="4" r:id="Rd57d1be917014bf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOVERNANCE" sheetId="5" r:id="R707328e9ae354a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5f33f163d7724253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_CONFIG" sheetId="2" r:id="Rfcbbe5b603004001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ASSUMPTIONS" sheetId="3" r:id="R5976e0601c7843e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_INPUT" sheetId="4" r:id="Rb0b61caaa08b4c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOVERNANCE" sheetId="5" r:id="Red28db0cab1042ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASA_INPUT" sheetId="6" r:id="Raf7aa51655fa459f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASA_GOVERNANCE" sheetId="7" r:id="R9a14e0f88ee54d4e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +24,7 @@
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,13 +46,33 @@
       <x:color rgb="FF0000FF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2747"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -75,7 +97,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -114,6 +136,33 @@
     <x:xf numFmtId="201" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -396,6 +445,14 @@
         <x:v>Không dùng lãi suất tiền gửi/cho vay để giả làm interbank ON.</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="28" t="str">
+        <x:v>CASA ACTUAL</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>Nếu Vnstock không có CASA/demand deposits, nhập CASA ACTUAL từ BCTC/IR/công bố chính thức tại sheet CASA_INPUT. Pipeline chỉ nhận DataType=ACTUAL + SourceURL hợp lệ và gắn lineage ACTUAL_MIXED_SOURCE.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -1858,4 +1915,594 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="42" t="str">
+        <x:v>CASA ACTUAL INPUT — NGUỒN CÔNG BỐ CHÍNH THỨC</x:v>
+      </x:c>
+      <x:c r="B1" s="42"/>
+      <x:c r="C1" s="42"/>
+      <x:c r="D1" s="42"/>
+      <x:c r="E1" s="42"/>
+      <x:c r="F1" s="42"/>
+      <x:c r="G1" s="42"/>
+      <x:c r="H1" s="42"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Ticker</x:v>
+      </x:c>
+      <x:c r="B3" s="34" t="str">
+        <x:v>Period</x:v>
+      </x:c>
+      <x:c r="C3" s="34" t="str">
+        <x:v>As Of Date</x:v>
+      </x:c>
+      <x:c r="D3" s="34" t="str">
+        <x:v>CASA</x:v>
+      </x:c>
+      <x:c r="E3" s="34" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+      <x:c r="F3" s="34" t="str">
+        <x:v>Source Name</x:v>
+      </x:c>
+      <x:c r="G3" s="34" t="str">
+        <x:v>Data Type</x:v>
+      </x:c>
+      <x:c r="H3" s="34" t="str">
+        <x:v>Instruction</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>VCB</x:v>
+      </x:c>
+      <x:c r="B4" s="39" t="str"/>
+      <x:c r="C4" s="40"/>
+      <x:c r="D4" s="41"/>
+      <x:c r="E4" s="39" t="str"/>
+      <x:c r="F4" s="39" t="str"/>
+      <x:c r="G4" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>BID</x:v>
+      </x:c>
+      <x:c r="B5" s="39" t="str"/>
+      <x:c r="C5" s="40"/>
+      <x:c r="D5" s="41"/>
+      <x:c r="E5" s="39" t="str"/>
+      <x:c r="F5" s="39" t="str"/>
+      <x:c r="G5" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>CTG</x:v>
+      </x:c>
+      <x:c r="B6" s="39" t="str"/>
+      <x:c r="C6" s="40"/>
+      <x:c r="D6" s="41"/>
+      <x:c r="E6" s="39" t="str"/>
+      <x:c r="F6" s="39" t="str"/>
+      <x:c r="G6" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>TCB</x:v>
+      </x:c>
+      <x:c r="B7" s="39" t="str"/>
+      <x:c r="C7" s="40"/>
+      <x:c r="D7" s="41"/>
+      <x:c r="E7" s="39" t="str"/>
+      <x:c r="F7" s="39" t="str"/>
+      <x:c r="G7" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>MBB</x:v>
+      </x:c>
+      <x:c r="B8" s="39" t="str"/>
+      <x:c r="C8" s="40"/>
+      <x:c r="D8" s="41"/>
+      <x:c r="E8" s="39" t="str"/>
+      <x:c r="F8" s="39" t="str"/>
+      <x:c r="G8" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>ACB</x:v>
+      </x:c>
+      <x:c r="B9" s="39" t="str"/>
+      <x:c r="C9" s="40"/>
+      <x:c r="D9" s="41"/>
+      <x:c r="E9" s="39" t="str"/>
+      <x:c r="F9" s="39" t="str"/>
+      <x:c r="G9" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>HDB</x:v>
+      </x:c>
+      <x:c r="B10" s="39" t="str"/>
+      <x:c r="C10" s="40"/>
+      <x:c r="D10" s="41"/>
+      <x:c r="E10" s="39" t="str"/>
+      <x:c r="F10" s="39" t="str"/>
+      <x:c r="G10" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>VPB</x:v>
+      </x:c>
+      <x:c r="B11" s="39" t="str"/>
+      <x:c r="C11" s="40"/>
+      <x:c r="D11" s="41"/>
+      <x:c r="E11" s="39" t="str"/>
+      <x:c r="F11" s="39" t="str"/>
+      <x:c r="G11" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>STB</x:v>
+      </x:c>
+      <x:c r="B12" s="39" t="str"/>
+      <x:c r="C12" s="40"/>
+      <x:c r="D12" s="41"/>
+      <x:c r="E12" s="39" t="str"/>
+      <x:c r="F12" s="39" t="str"/>
+      <x:c r="G12" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>VIB</x:v>
+      </x:c>
+      <x:c r="B13" s="39" t="str"/>
+      <x:c r="C13" s="40"/>
+      <x:c r="D13" s="41"/>
+      <x:c r="E13" s="39" t="str"/>
+      <x:c r="F13" s="39" t="str"/>
+      <x:c r="G13" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>SHB</x:v>
+      </x:c>
+      <x:c r="B14" s="39" t="str"/>
+      <x:c r="C14" s="40"/>
+      <x:c r="D14" s="41"/>
+      <x:c r="E14" s="39" t="str"/>
+      <x:c r="F14" s="39" t="str"/>
+      <x:c r="G14" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>TPB</x:v>
+      </x:c>
+      <x:c r="B15" s="39" t="str"/>
+      <x:c r="C15" s="40"/>
+      <x:c r="D15" s="41"/>
+      <x:c r="E15" s="39" t="str"/>
+      <x:c r="F15" s="39" t="str"/>
+      <x:c r="G15" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>LPB</x:v>
+      </x:c>
+      <x:c r="B16" s="39" t="str"/>
+      <x:c r="C16" s="40"/>
+      <x:c r="D16" s="41"/>
+      <x:c r="E16" s="39" t="str"/>
+      <x:c r="F16" s="39" t="str"/>
+      <x:c r="G16" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>OCB</x:v>
+      </x:c>
+      <x:c r="B17" s="39" t="str"/>
+      <x:c r="C17" s="40"/>
+      <x:c r="D17" s="41"/>
+      <x:c r="E17" s="39" t="str"/>
+      <x:c r="F17" s="39" t="str"/>
+      <x:c r="G17" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>MSB</x:v>
+      </x:c>
+      <x:c r="B18" s="39" t="str"/>
+      <x:c r="C18" s="40"/>
+      <x:c r="D18" s="41"/>
+      <x:c r="E18" s="39" t="str"/>
+      <x:c r="F18" s="39" t="str"/>
+      <x:c r="G18" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>SSB</x:v>
+      </x:c>
+      <x:c r="B19" s="39" t="str"/>
+      <x:c r="C19" s="40"/>
+      <x:c r="D19" s="41"/>
+      <x:c r="E19" s="39" t="str"/>
+      <x:c r="F19" s="39" t="str"/>
+      <x:c r="G19" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>EIB</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="str"/>
+      <x:c r="C20" s="40"/>
+      <x:c r="D20" s="41"/>
+      <x:c r="E20" s="39" t="str"/>
+      <x:c r="F20" s="39" t="str"/>
+      <x:c r="G20" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>NAB</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="str"/>
+      <x:c r="C21" s="40"/>
+      <x:c r="D21" s="41"/>
+      <x:c r="E21" s="39" t="str"/>
+      <x:c r="F21" s="39" t="str"/>
+      <x:c r="G21" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>KLB</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="str"/>
+      <x:c r="C22" s="40"/>
+      <x:c r="D22" s="41"/>
+      <x:c r="E22" s="39" t="str"/>
+      <x:c r="F22" s="39" t="str"/>
+      <x:c r="G22" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>BAB</x:v>
+      </x:c>
+      <x:c r="B23" s="39" t="str"/>
+      <x:c r="C23" s="40"/>
+      <x:c r="D23" s="41"/>
+      <x:c r="E23" s="39" t="str"/>
+      <x:c r="F23" s="39" t="str"/>
+      <x:c r="G23" s="39" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Nhập CASA công bố chính thức; Source URL bắt buộc. Có thể nhập 0.35 hoặc 35.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="42" t="str">
+        <x:v>CASA DATA ACQUISITION &amp; LINEAGE GOVERNANCE</x:v>
+      </x:c>
+      <x:c r="B1" s="42"/>
+      <x:c r="C1" s="42"/>
+      <x:c r="D1" s="42"/>
+      <x:c r="E1" s="42"/>
+      <x:c r="F1" s="42"/>
+      <x:c r="G1" s="42"/>
+      <x:c r="H1" s="42"/>
+      <x:c r="I1" s="42"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="B3" s="34" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="C3" s="34" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="D3" s="34" t="str">
+        <x:v>Accepted as ACTUAL?</x:v>
+      </x:c>
+      <x:c r="E3" s="34" t="str">
+        <x:v>CASASource</x:v>
+      </x:c>
+      <x:c r="F3" s="34" t="str">
+        <x:v>Stress lineage if 5/5 actual</x:v>
+      </x:c>
+      <x:c r="G3" s="34" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="H3" s="34" t="str">
+        <x:v>Fallback action</x:v>
+      </x:c>
+      <x:c r="I3" s="34" t="str">
+        <x:v>Audit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Vnstock financial_health</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Direct reported CASA</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>DIRECT_FINANCIAL_HEALTH</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>BRONZE</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>0≤CASA≤100%</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Next source</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>bank_metrics.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Vnstock ratio</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Direct reported CASA</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>DIRECT_RATIO</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>BRONZE</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>0≤CASA≤100%</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Next source</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>bank_metrics.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Vnstock balance sheet</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Demand/non-term deposits ÷ customer deposits</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>DERIVED_BALANCE_SHEET</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>BRONZE</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Numerator &amp; denominator both actual</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Next source</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>bank_metrics.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>BCTC / IR / official disclosure</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>CASA_INPUT → casa_actual.csv</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>ACTUAL_PUBLIC_SOURCE</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>ACTUAL_MIXED_SOURCE</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>DataType=ACTUAL + SourceURL + 0≤CASA≤100%</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Use model assumption only for CASA</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>CASA_INPUT + casa_actual.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Model assumption</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>bank_assumptions.csv</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>MODEL_ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>HYBRID</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Never shown as ACTUAL</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Use only inside stress model</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>bank_stress.csv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Accumulate interbank ACTUAL history and governed forecast tiers
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Liquidity_Master.xlsx
+++ b/Vietnam_Banking_Liquidity_Master.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2ae49af500274603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_CONFIG" sheetId="2" r:id="Rcfc855fe9d264dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ASSUMPTIONS" sheetId="3" r:id="R27e109e345d2410c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_INPUT" sheetId="4" r:id="R663038df29de4b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOVERNANCE" sheetId="5" r:id="Rc7e471be07624eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASA_INPUT" sheetId="6" r:id="Rbf0804729a744a42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASA_GOVERNANCE" sheetId="7" r:id="R670c43b754ed4080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4e0f3ea3af6c4b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MODEL_CONFIG" sheetId="2" r:id="R70534588fe1c487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ASSUMPTIONS" sheetId="3" r:id="Rb9e92bb61c7946df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_INPUT" sheetId="4" r:id="R63fd5416cc2347b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOVERNANCE" sheetId="5" r:id="Rfeddb3c5464e4f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASA_INPUT" sheetId="6" r:id="R9076d21e3f45456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASA_GOVERNANCE" sheetId="7" r:id="Ra7759764cf13482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INTERBANK_HISTORY" sheetId="8" r:id="R431f5f2a4b8b478f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +54,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +91,21 @@
         <x:fgColor rgb="FFFFFF00"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2747"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -98,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -165,6 +181,25 @@
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -463,6 +498,14 @@
         <x:v>Đã nạp CASA 30/06/2026 cho đủ 20 ngân hàng từ bảng VietNamNet tổng hợp BCTC bán niên. Pipeline gắn ACTUAL_PUBLIC_SOURCE và có thể được thay thế bởi CASA mới hơn trong data/casa_actual.csv.</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="28" t="str">
+        <x:v>Interbank history</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>Mỗi refresh append ACTUAL ON vào data/interbank_history.csv rồi deduplicate theo ngày. 0–39 quan sát: actual-only; 40–79: exploratory/LOW confidence; &gt;=80: production-eligible.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -692,6 +735,46 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="F13" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="27" t="str">
+        <x:v>Minimum Interbank exploratory observations</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C14" s="27" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D14" s="27" t="str">
+        <x:v>Cho phép forecast exploratory, LOW confidence</x:v>
+      </x:c>
+      <x:c r="E14" s="27" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F14" s="27" t="str">
+        <x:v>Không dùng như production forecast</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="27" t="str">
+        <x:v>Minimum Interbank production observations</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>ASSUMPTION</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="str">
+        <x:v>Ngưỡng lịch sử ON để forecast production</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F15" s="27" t="str">
+        <x:v>Vẫn phải vượt naive benchmark</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2715,4 +2798,243 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="52" t="str">
+        <x:v>INTERBANK ON — HISTORY ACCUMULATION &amp; FORECAST GOVERNANCE</x:v>
+      </x:c>
+      <x:c r="B1" s="52"/>
+      <x:c r="C1" s="52"/>
+      <x:c r="D1" s="52"/>
+      <x:c r="E1" s="52"/>
+      <x:c r="F1" s="52"/>
+      <x:c r="G1" s="52"/>
+      <x:c r="H1" s="52"/>
+      <x:c r="I1" s="52"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="51" t="str">
+        <x:v>Layer</x:v>
+      </x:c>
+      <x:c r="B3" s="51" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="C3" s="51" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="D3" s="51" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="E3" s="51" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="F3" s="51" t="str">
+        <x:v>Threshold</x:v>
+      </x:c>
+      <x:c r="G3" s="51" t="str">
+        <x:v>Forecast Tier</x:v>
+      </x:c>
+      <x:c r="H3" s="51" t="str">
+        <x:v>Can overwrite history?</x:v>
+      </x:c>
+      <x:c r="I3" s="51" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>History</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Append + deduplicate by date</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Existing interbank_history.csv</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Preserved ACTUAL history</x:v>
+      </x:c>
+      <x:c r="E4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Refresh failure never deletes old ACTUAL observations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Acquisition</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Fresh Vnstock ON</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>interbank_rate / interest_rate</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>New ACTUAL observations</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Only same-date replace</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Fresh Bronze supersedes stale same-date history</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Manual/Public</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Source-cited ACTUAL</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>interbank_manual.csv</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Validated ACTUAL observations</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Only same-date replace</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Highest duplicate-date priority</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Forecast</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Actual only</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>0–39 observations</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>No forecast</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>&lt;40</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>ACTUAL_ONLY</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Chart actual; accumulate more history</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Forecast</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Exploratory</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>40–79 observations</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Forecast with warning</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>40–79</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>EXPLORATORY</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>LOW confidence; not production</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Forecast</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Production eligibility</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>&gt;=80 observations</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Governed forecast</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>&gt;=80</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>PRODUCTION</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>ARIMA still must beat naive benchmark</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>